<commit_message>
# Updated list of models
</commit_message>
<xml_diff>
--- a/List of GSM-Converted Kinetic Models.xlsx
+++ b/List of GSM-Converted Kinetic Models.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\MyProjects\kinmodre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C58B999-7DEB-4C58-8420-BC79EA2AA638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF689A9-50D7-4DA3-BDEC-B0A0D38963E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B4C7D942-9A2E-4284-ADB5-B7C4CF7DD1B1}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="207">
   <si>
     <t>e_coli_core</t>
   </si>
@@ -643,6 +643,21 @@
   </si>
   <si>
     <t>Reference</t>
+  </si>
+  <si>
+    <t>GSM File (in GSM folder)</t>
+  </si>
+  <si>
+    <t>ASM File (in asm folder)</t>
+  </si>
+  <si>
+    <t>ODE Script File (in odescripts folder)</t>
+  </si>
+  <si>
+    <t>ODE Script File (in GSM-odescripts folder)</t>
+  </si>
+  <si>
+    <t>OK</t>
   </si>
 </sst>
 </file>
@@ -733,7 +748,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -769,6 +784,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1106,17 +1127,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC6CDDD6-2BE3-467B-8E7F-78A96156F001}">
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:K109"/>
   <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22.81640625" style="7" customWidth="1"/>
-    <col min="2" max="2" width="63.6328125" style="7" customWidth="1"/>
-    <col min="3" max="5" width="14" style="8" customWidth="1"/>
-    <col min="6" max="6" width="14.26953125" style="7" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" style="1"/>
+    <col min="2" max="2" width="46.1796875" style="7" customWidth="1"/>
+    <col min="3" max="5" width="14" style="8" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="10.26953125" style="7" hidden="1" customWidth="1"/>
+    <col min="7" max="10" width="21.6328125" style="7" customWidth="1"/>
+    <col min="11" max="11" width="12.36328125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="21.6328125" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" ht="32" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>193</v>
       </c>
@@ -1135,8 +1159,20 @@
       <c r="F1" s="3" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G1" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1155,8 +1191,27 @@
       <c r="F2" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G2" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A2,".xml"),_xlfn.CONCAT(A2,".xml"))</f>
+        <v>e_coli_core.xml</v>
+      </c>
+      <c r="H2" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A2,".modelspec"),_xlfn.CONCAT(A2,".modelspec"))</f>
+        <v>e_coli_core.modelspec</v>
+      </c>
+      <c r="I2" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A2,".py"),_xlfn.CONCAT(A2,".py"))</f>
+        <v>e_coli_core.py</v>
+      </c>
+      <c r="J2" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A2,".py"),_xlfn.CONCAT(A2,".py"))</f>
+        <v>e_coli_core.py</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1175,8 +1230,27 @@
       <c r="F3" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G3" s="14" t="str">
+        <f t="shared" ref="G3:G66" si="0">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A3,".xml"),_xlfn.CONCAT(A3,".xml"))</f>
+        <v>iAB_RBC_283.xml</v>
+      </c>
+      <c r="H3" s="14" t="str">
+        <f t="shared" ref="H3:H66" si="1">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A3,".modelspec"),_xlfn.CONCAT(A3,".modelspec"))</f>
+        <v>iAB_RBC_283.modelspec</v>
+      </c>
+      <c r="I3" s="14" t="str">
+        <f t="shared" ref="I3:I66" si="2">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A3,".py"),_xlfn.CONCAT(A3,".py"))</f>
+        <v>iAB_RBC_283.py</v>
+      </c>
+      <c r="J3" s="14" t="str">
+        <f t="shared" ref="J3:J66" si="3">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A3,".py"),_xlfn.CONCAT(A3,".py"))</f>
+        <v>iAB_RBC_283.py</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -1195,8 +1269,27 @@
       <c r="F4" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G4" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iAF1260.xml</v>
+      </c>
+      <c r="H4" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iAF1260.modelspec</v>
+      </c>
+      <c r="I4" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A4,".py"),_xlfn.CONCAT(A4,".py"))</f>
+        <v>iAF1260.py</v>
+      </c>
+      <c r="J4" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iAF1260.py</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
@@ -1215,8 +1308,27 @@
       <c r="F5" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G5" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iAF1260b.xml</v>
+      </c>
+      <c r="H5" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iAF1260b.modelspec</v>
+      </c>
+      <c r="I5" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iAF1260b.py</v>
+      </c>
+      <c r="J5" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iAF1260b.py</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
@@ -1235,8 +1347,27 @@
       <c r="F6" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G6" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iAF692.xml</v>
+      </c>
+      <c r="H6" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iAF692.modelspec</v>
+      </c>
+      <c r="I6" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iAF692.py</v>
+      </c>
+      <c r="J6" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iAF692.py</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
@@ -1255,8 +1386,27 @@
       <c r="F7" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G7" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iAF987.xml</v>
+      </c>
+      <c r="H7" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iAF987.modelspec</v>
+      </c>
+      <c r="I7" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iAF987.py</v>
+      </c>
+      <c r="J7" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iAF987.py</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
@@ -1275,8 +1425,27 @@
       <c r="F8" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G8" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A8,".xml"),_xlfn.CONCAT(A8,".xml"))</f>
+        <v>iAM_Pb448.xml</v>
+      </c>
+      <c r="H8" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iAM_Pb448.modelspec</v>
+      </c>
+      <c r="I8" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iAM_Pb448.py</v>
+      </c>
+      <c r="J8" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iAM_Pb448.py</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
@@ -1295,8 +1464,27 @@
       <c r="F9" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G9" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iAM_Pc455.xml</v>
+      </c>
+      <c r="H9" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iAM_Pc455.modelspec</v>
+      </c>
+      <c r="I9" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A9,".py"),_xlfn.CONCAT(A9,".py"))</f>
+        <v>iAM_Pc455.py</v>
+      </c>
+      <c r="J9" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iAM_Pc455.py</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
@@ -1315,8 +1503,27 @@
       <c r="F10" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G10" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iAM_Pf480.xml</v>
+      </c>
+      <c r="H10" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iAM_Pf480.modelspec</v>
+      </c>
+      <c r="I10" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A10,".py"),_xlfn.CONCAT(A10,".py"))</f>
+        <v>iAM_Pf480.py</v>
+      </c>
+      <c r="J10" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A10,".py"),_xlfn.CONCAT(A10,".py"))</f>
+        <v>iAM_Pf480.py</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>16</v>
       </c>
@@ -1335,8 +1542,27 @@
       <c r="F11" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G11" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A11,".xml"),_xlfn.CONCAT(A11,".xml"))</f>
+        <v>iAM_Pk459.xml</v>
+      </c>
+      <c r="H11" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A11,".modelspec"),_xlfn.CONCAT(A11,".modelspec"))</f>
+        <v>iAM_Pk459.modelspec</v>
+      </c>
+      <c r="I11" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iAM_Pk459.py</v>
+      </c>
+      <c r="J11" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iAM_Pk459.py</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>18</v>
       </c>
@@ -1355,8 +1581,27 @@
       <c r="F12" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G12" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iAM_Pv461.xml</v>
+      </c>
+      <c r="H12" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iAM_Pv461.modelspec</v>
+      </c>
+      <c r="I12" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A12,".py"),_xlfn.CONCAT(A12,".py"))</f>
+        <v>iAM_Pv461.py</v>
+      </c>
+      <c r="J12" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iAM_Pv461.py</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>20</v>
       </c>
@@ -1375,8 +1620,27 @@
       <c r="F13" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G13" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iAPECO1_1312.xml</v>
+      </c>
+      <c r="H13" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iAPECO1_1312.modelspec</v>
+      </c>
+      <c r="I13" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A13,".py"),_xlfn.CONCAT(A13,".py"))</f>
+        <v>iAPECO1_1312.py</v>
+      </c>
+      <c r="J13" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A13,".py"),_xlfn.CONCAT(A13,".py"))</f>
+        <v>iAPECO1_1312.py</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A14" s="4" t="s">
         <v>22</v>
       </c>
@@ -1395,8 +1659,27 @@
       <c r="F14" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G14" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iAT_PLT_636.xml</v>
+      </c>
+      <c r="H14" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iAT_PLT_636.modelspec</v>
+      </c>
+      <c r="I14" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A14,".py"),_xlfn.CONCAT(A14,".py"))</f>
+        <v>iAT_PLT_636.py</v>
+      </c>
+      <c r="J14" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iAT_PLT_636.py</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A15" s="4" t="s">
         <v>23</v>
       </c>
@@ -1415,8 +1698,27 @@
       <c r="F15" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G15" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iB21_1397.xml</v>
+      </c>
+      <c r="H15" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iB21_1397.modelspec</v>
+      </c>
+      <c r="I15" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A15,".py"),_xlfn.CONCAT(A15,".py"))</f>
+        <v>iB21_1397.py</v>
+      </c>
+      <c r="J15" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A15,".py"),_xlfn.CONCAT(A15,".py"))</f>
+        <v>iB21_1397.py</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A16" s="4" t="s">
         <v>25</v>
       </c>
@@ -1435,8 +1737,27 @@
       <c r="F16" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G16" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iBWG_1329.xml</v>
+      </c>
+      <c r="H16" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iBWG_1329.modelspec</v>
+      </c>
+      <c r="I16" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iBWG_1329.py</v>
+      </c>
+      <c r="J16" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A16,".py"),_xlfn.CONCAT(A16,".py"))</f>
+        <v>iBWG_1329.py</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A17" s="4" t="s">
         <v>27</v>
       </c>
@@ -1455,8 +1776,27 @@
       <c r="F17" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G17" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>ic_1306.xml</v>
+      </c>
+      <c r="H17" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>ic_1306.modelspec</v>
+      </c>
+      <c r="I17" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A17,".py"),_xlfn.CONCAT(A17,".py"))</f>
+        <v>ic_1306.py</v>
+      </c>
+      <c r="J17" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>ic_1306.py</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A18" s="4" t="s">
         <v>29</v>
       </c>
@@ -1475,8 +1815,27 @@
       <c r="F18" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G18" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A18,".xml"),_xlfn.CONCAT(A18,".xml"))</f>
+        <v>iCHOv1.xml</v>
+      </c>
+      <c r="H18" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iCHOv1.modelspec</v>
+      </c>
+      <c r="I18" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iCHOv1.py</v>
+      </c>
+      <c r="J18" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iCHOv1.py</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
         <v>31</v>
       </c>
@@ -1495,8 +1854,28 @@
       <c r="F19" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G19" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iCHOv1_DG44.xml</v>
+      </c>
+      <c r="H19" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A19,".modelspec"),_xlfn.CONCAT(A19,".modelspec"))</f>
+        <v>iCHOv1_DG44.modelspec</v>
+      </c>
+      <c r="I19" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iCHOv1_DG44.py</v>
+      </c>
+      <c r="J19" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iCHOv1_DG44.py</v>
+      </c>
+      <c r="K19" s="13" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/Minionnick/kinmodre/tree/main/asm/",A19,".modelspec"),_xlfn.CONCAT(A19,".modelspec"))</f>
+        <v>iCHOv1_DG44.modelspec</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
@@ -1515,8 +1894,28 @@
       <c r="F20" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G20" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iCN718.xml</v>
+      </c>
+      <c r="H20" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iCN718.modelspec</v>
+      </c>
+      <c r="I20" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iCN718.py</v>
+      </c>
+      <c r="J20" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iCN718.py</v>
+      </c>
+      <c r="K20" s="13" t="str">
+        <f t="shared" ref="K20:K50" si="4">HYPERLINK(_xlfn.CONCAT("https://github.com/Minionnick/kinmodre/tree/main/asm/",A20,".modelspec"),_xlfn.CONCAT(A20,".modelspec"))</f>
+        <v>iCN718.modelspec</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A21" s="4" t="s">
         <v>34</v>
       </c>
@@ -1535,8 +1934,28 @@
       <c r="F21" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G21" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iCN900.xml</v>
+      </c>
+      <c r="H21" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iCN900.modelspec</v>
+      </c>
+      <c r="I21" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A21,".py"),_xlfn.CONCAT(A21,".py"))</f>
+        <v>iCN900.py</v>
+      </c>
+      <c r="J21" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A21,".py"),_xlfn.CONCAT(A21,".py"))</f>
+        <v>iCN900.py</v>
+      </c>
+      <c r="K21" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iCN900.modelspec</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
         <v>36</v>
       </c>
@@ -1555,8 +1974,28 @@
       <c r="F22" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G22" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iE2348C_1286.xml</v>
+      </c>
+      <c r="H22" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iE2348C_1286.modelspec</v>
+      </c>
+      <c r="I22" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iE2348C_1286.py</v>
+      </c>
+      <c r="J22" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A22,".py"),_xlfn.CONCAT(A22,".py"))</f>
+        <v>iE2348C_1286.py</v>
+      </c>
+      <c r="K22" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iE2348C_1286.modelspec</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A23" s="4" t="s">
         <v>38</v>
       </c>
@@ -1575,8 +2014,28 @@
       <c r="F23" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G23" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A23,".xml"),_xlfn.CONCAT(A23,".xml"))</f>
+        <v>iEC042_1314.xml</v>
+      </c>
+      <c r="H23" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iEC042_1314.modelspec</v>
+      </c>
+      <c r="I23" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A23,".py"),_xlfn.CONCAT(A23,".py"))</f>
+        <v>iEC042_1314.py</v>
+      </c>
+      <c r="J23" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEC042_1314.py</v>
+      </c>
+      <c r="K23" s="13" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/Minionnick/kinmodre/tree/main/asm/",A23,".modelspec"),_xlfn.CONCAT(A23,".modelspec"))</f>
+        <v>iEC042_1314.modelspec</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A24" s="4" t="s">
         <v>40</v>
       </c>
@@ -1595,8 +2054,28 @@
       <c r="F24" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G24" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A24,".xml"),_xlfn.CONCAT(A24,".xml"))</f>
+        <v>iEC1344_C.xml</v>
+      </c>
+      <c r="H24" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A24,".modelspec"),_xlfn.CONCAT(A24,".modelspec"))</f>
+        <v>iEC1344_C.modelspec</v>
+      </c>
+      <c r="I24" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iEC1344_C.py</v>
+      </c>
+      <c r="J24" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEC1344_C.py</v>
+      </c>
+      <c r="K24" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iEC1344_C.modelspec</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A25" s="4" t="s">
         <v>42</v>
       </c>
@@ -1615,8 +2094,28 @@
       <c r="F25" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G25" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iEC1349_Crooks.xml</v>
+      </c>
+      <c r="H25" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iEC1349_Crooks.modelspec</v>
+      </c>
+      <c r="I25" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iEC1349_Crooks.py</v>
+      </c>
+      <c r="J25" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEC1349_Crooks.py</v>
+      </c>
+      <c r="K25" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iEC1349_Crooks.modelspec</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
         <v>44</v>
       </c>
@@ -1635,8 +2134,28 @@
       <c r="F26" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G26" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iEC1356_Bl21DE3.xml</v>
+      </c>
+      <c r="H26" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iEC1356_Bl21DE3.modelspec</v>
+      </c>
+      <c r="I26" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iEC1356_Bl21DE3.py</v>
+      </c>
+      <c r="J26" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A26,".py"),_xlfn.CONCAT(A26,".py"))</f>
+        <v>iEC1356_Bl21DE3.py</v>
+      </c>
+      <c r="K26" s="13" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/Minionnick/kinmodre/tree/main/asm/",A26,".modelspec"),_xlfn.CONCAT(A26,".modelspec"))</f>
+        <v>iEC1356_Bl21DE3.modelspec</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A27" s="4" t="s">
         <v>45</v>
       </c>
@@ -1655,8 +2174,28 @@
       <c r="F27" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G27" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iEC1364_W.xml</v>
+      </c>
+      <c r="H27" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A27,".modelspec"),_xlfn.CONCAT(A27,".modelspec"))</f>
+        <v>iEC1364_W.modelspec</v>
+      </c>
+      <c r="I27" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iEC1364_W.py</v>
+      </c>
+      <c r="J27" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEC1364_W.py</v>
+      </c>
+      <c r="K27" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iEC1364_W.modelspec</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
         <v>47</v>
       </c>
@@ -1675,8 +2214,28 @@
       <c r="F28" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G28" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iEC1368_DH5a.xml</v>
+      </c>
+      <c r="H28" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A28,".modelspec"),_xlfn.CONCAT(A28,".modelspec"))</f>
+        <v>iEC1368_DH5a.modelspec</v>
+      </c>
+      <c r="I28" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iEC1368_DH5a.py</v>
+      </c>
+      <c r="J28" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A28,".py"),_xlfn.CONCAT(A28,".py"))</f>
+        <v>iEC1368_DH5a.py</v>
+      </c>
+      <c r="K28" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iEC1368_DH5a.modelspec</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
         <v>49</v>
       </c>
@@ -1695,8 +2254,28 @@
       <c r="F29" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G29" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iEC1372_W3110.xml</v>
+      </c>
+      <c r="H29" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iEC1372_W3110.modelspec</v>
+      </c>
+      <c r="I29" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iEC1372_W3110.py</v>
+      </c>
+      <c r="J29" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEC1372_W3110.py</v>
+      </c>
+      <c r="K29" s="13" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/Minionnick/kinmodre/tree/main/asm/",A29,".modelspec"),_xlfn.CONCAT(A29,".modelspec"))</f>
+        <v>iEC1372_W3110.modelspec</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A30" s="4" t="s">
         <v>51</v>
       </c>
@@ -1715,8 +2294,28 @@
       <c r="F30" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G30" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iEC55989_1330.xml</v>
+      </c>
+      <c r="H30" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iEC55989_1330.modelspec</v>
+      </c>
+      <c r="I30" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iEC55989_1330.py</v>
+      </c>
+      <c r="J30" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEC55989_1330.py</v>
+      </c>
+      <c r="K30" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iEC55989_1330.modelspec</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A31" s="4" t="s">
         <v>53</v>
       </c>
@@ -1735,8 +2334,28 @@
       <c r="F31" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G31" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A31,".xml"),_xlfn.CONCAT(A31,".xml"))</f>
+        <v>iECABU_c1320.xml</v>
+      </c>
+      <c r="H31" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A31,".modelspec"),_xlfn.CONCAT(A31,".modelspec"))</f>
+        <v>iECABU_c1320.modelspec</v>
+      </c>
+      <c r="I31" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECABU_c1320.py</v>
+      </c>
+      <c r="J31" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECABU_c1320.py</v>
+      </c>
+      <c r="K31" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECABU_c1320.modelspec</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
         <v>55</v>
       </c>
@@ -1755,8 +2374,28 @@
       <c r="F32" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G32" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECB_1328.xml</v>
+      </c>
+      <c r="H32" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A32,".modelspec"),_xlfn.CONCAT(A32,".modelspec"))</f>
+        <v>iECB_1328.modelspec</v>
+      </c>
+      <c r="I32" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECB_1328.py</v>
+      </c>
+      <c r="J32" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A32,".py"),_xlfn.CONCAT(A32,".py"))</f>
+        <v>iECB_1328.py</v>
+      </c>
+      <c r="K32" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECB_1328.modelspec</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A33" s="4" t="s">
         <v>57</v>
       </c>
@@ -1775,8 +2414,28 @@
       <c r="F33" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G33" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECBD_1354.xml</v>
+      </c>
+      <c r="H33" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECBD_1354.modelspec</v>
+      </c>
+      <c r="I33" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECBD_1354.py</v>
+      </c>
+      <c r="J33" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A33,".py"),_xlfn.CONCAT(A33,".py"))</f>
+        <v>iECBD_1354.py</v>
+      </c>
+      <c r="K33" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECBD_1354.modelspec</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A34" s="4" t="s">
         <v>59</v>
       </c>
@@ -1795,8 +2454,28 @@
       <c r="F34" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G34" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A34,".xml"),_xlfn.CONCAT(A34,".xml"))</f>
+        <v>iECD_1391.xml</v>
+      </c>
+      <c r="H34" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECD_1391.modelspec</v>
+      </c>
+      <c r="I34" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A34,".py"),_xlfn.CONCAT(A34,".py"))</f>
+        <v>iECD_1391.py</v>
+      </c>
+      <c r="J34" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A34,".py"),_xlfn.CONCAT(A34,".py"))</f>
+        <v>iECD_1391.py</v>
+      </c>
+      <c r="K34" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECD_1391.modelspec</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A35" s="4" t="s">
         <v>60</v>
       </c>
@@ -1815,8 +2494,28 @@
       <c r="F35" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G35" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECDH10B_1368.xml</v>
+      </c>
+      <c r="H35" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A35,".modelspec"),_xlfn.CONCAT(A35,".modelspec"))</f>
+        <v>iECDH10B_1368.modelspec</v>
+      </c>
+      <c r="I35" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECDH10B_1368.py</v>
+      </c>
+      <c r="J35" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECDH10B_1368.py</v>
+      </c>
+      <c r="K35" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECDH10B_1368.modelspec</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A36" s="4" t="s">
         <v>62</v>
       </c>
@@ -1835,8 +2534,28 @@
       <c r="F36" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G36" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iEcDH1_1363.xml</v>
+      </c>
+      <c r="H36" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iEcDH1_1363.modelspec</v>
+      </c>
+      <c r="I36" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A36,".py"),_xlfn.CONCAT(A36,".py"))</f>
+        <v>iEcDH1_1363.py</v>
+      </c>
+      <c r="J36" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEcDH1_1363.py</v>
+      </c>
+      <c r="K36" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iEcDH1_1363.modelspec</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A37" s="4" t="s">
         <v>64</v>
       </c>
@@ -1855,8 +2574,28 @@
       <c r="F37" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G37" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECDH1ME8569_1439.xml</v>
+      </c>
+      <c r="H37" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECDH1ME8569_1439.modelspec</v>
+      </c>
+      <c r="I37" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A37,".py"),_xlfn.CONCAT(A37,".py"))</f>
+        <v>iECDH1ME8569_1439.py</v>
+      </c>
+      <c r="J37" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECDH1ME8569_1439.py</v>
+      </c>
+      <c r="K37" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECDH1ME8569_1439.modelspec</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A38" s="4" t="s">
         <v>65</v>
       </c>
@@ -1875,8 +2614,28 @@
       <c r="F38" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G38" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iEcE24377_1341.xml</v>
+      </c>
+      <c r="H38" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iEcE24377_1341.modelspec</v>
+      </c>
+      <c r="I38" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iEcE24377_1341.py</v>
+      </c>
+      <c r="J38" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEcE24377_1341.py</v>
+      </c>
+      <c r="K38" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iEcE24377_1341.modelspec</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A39" s="4" t="s">
         <v>67</v>
       </c>
@@ -1895,8 +2654,28 @@
       <c r="F39" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G39" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECED1_1282.xml</v>
+      </c>
+      <c r="H39" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECED1_1282.modelspec</v>
+      </c>
+      <c r="I39" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECED1_1282.py</v>
+      </c>
+      <c r="J39" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECED1_1282.py</v>
+      </c>
+      <c r="K39" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECED1_1282.modelspec</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A40" s="4" t="s">
         <v>69</v>
       </c>
@@ -1915,8 +2694,28 @@
       <c r="F40" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G40" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A40,".xml"),_xlfn.CONCAT(A40,".xml"))</f>
+        <v>iECH74115_1262.xml</v>
+      </c>
+      <c r="H40" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECH74115_1262.modelspec</v>
+      </c>
+      <c r="I40" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECH74115_1262.py</v>
+      </c>
+      <c r="J40" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECH74115_1262.py</v>
+      </c>
+      <c r="K40" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECH74115_1262.modelspec</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A41" s="4" t="s">
         <v>71</v>
       </c>
@@ -1935,8 +2734,28 @@
       <c r="F41" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G41" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iEcHS_1320.xml</v>
+      </c>
+      <c r="H41" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iEcHS_1320.modelspec</v>
+      </c>
+      <c r="I41" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iEcHS_1320.py</v>
+      </c>
+      <c r="J41" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEcHS_1320.py</v>
+      </c>
+      <c r="K41" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iEcHS_1320.modelspec</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A42" s="4" t="s">
         <v>73</v>
       </c>
@@ -1955,8 +2774,28 @@
       <c r="F42" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G42" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A42,".xml"),_xlfn.CONCAT(A42,".xml"))</f>
+        <v>iECIAI1_1343.xml</v>
+      </c>
+      <c r="H42" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECIAI1_1343.modelspec</v>
+      </c>
+      <c r="I42" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A42,".py"),_xlfn.CONCAT(A42,".py"))</f>
+        <v>iECIAI1_1343.py</v>
+      </c>
+      <c r="J42" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A42,".py"),_xlfn.CONCAT(A42,".py"))</f>
+        <v>iECIAI1_1343.py</v>
+      </c>
+      <c r="K42" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECIAI1_1343.modelspec</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A43" s="4" t="s">
         <v>75</v>
       </c>
@@ -1975,8 +2814,28 @@
       <c r="F43" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G43" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECIAI39_1322.xml</v>
+      </c>
+      <c r="H43" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECIAI39_1322.modelspec</v>
+      </c>
+      <c r="I43" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECIAI39_1322.py</v>
+      </c>
+      <c r="J43" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECIAI39_1322.py</v>
+      </c>
+      <c r="K43" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECIAI39_1322.modelspec</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A44" s="4" t="s">
         <v>77</v>
       </c>
@@ -1995,8 +2854,28 @@
       <c r="F44" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G44" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECNA114_1301.xml</v>
+      </c>
+      <c r="H44" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECNA114_1301.modelspec</v>
+      </c>
+      <c r="I44" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECNA114_1301.py</v>
+      </c>
+      <c r="J44" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A44,".py"),_xlfn.CONCAT(A44,".py"))</f>
+        <v>iECNA114_1301.py</v>
+      </c>
+      <c r="K44" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECNA114_1301.modelspec</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A45" s="4" t="s">
         <v>79</v>
       </c>
@@ -2015,8 +2894,28 @@
       <c r="F45" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G45" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECO103_1326.xml</v>
+      </c>
+      <c r="H45" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECO103_1326.modelspec</v>
+      </c>
+      <c r="I45" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECO103_1326.py</v>
+      </c>
+      <c r="J45" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECO103_1326.py</v>
+      </c>
+      <c r="K45" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECO103_1326.modelspec</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A46" s="4" t="s">
         <v>81</v>
       </c>
@@ -2035,8 +2934,28 @@
       <c r="F46" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G46" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A46,".xml"),_xlfn.CONCAT(A46,".xml"))</f>
+        <v>iECO111_1330.xml</v>
+      </c>
+      <c r="H46" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECO111_1330.modelspec</v>
+      </c>
+      <c r="I46" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECO111_1330.py</v>
+      </c>
+      <c r="J46" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A46,".py"),_xlfn.CONCAT(A46,".py"))</f>
+        <v>iECO111_1330.py</v>
+      </c>
+      <c r="K46" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECO111_1330.modelspec</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A47" s="4" t="s">
         <v>83</v>
       </c>
@@ -2055,8 +2974,28 @@
       <c r="F47" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G47" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A47,".xml"),_xlfn.CONCAT(A47,".xml"))</f>
+        <v>iECO26_1355.xml</v>
+      </c>
+      <c r="H47" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECO26_1355.modelspec</v>
+      </c>
+      <c r="I47" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECO26_1355.py</v>
+      </c>
+      <c r="J47" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECO26_1355.py</v>
+      </c>
+      <c r="K47" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECO26_1355.modelspec</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A48" s="4" t="s">
         <v>85</v>
       </c>
@@ -2075,8 +3014,28 @@
       <c r="F48" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G48" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECOK1_1307.xml</v>
+      </c>
+      <c r="H48" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECOK1_1307.modelspec</v>
+      </c>
+      <c r="I48" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECOK1_1307.py</v>
+      </c>
+      <c r="J48" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECOK1_1307.py</v>
+      </c>
+      <c r="K48" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECOK1_1307.modelspec</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A49" s="4" t="s">
         <v>87</v>
       </c>
@@ -2095,8 +3054,28 @@
       <c r="F49" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G49" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A49,".xml"),_xlfn.CONCAT(A49,".xml"))</f>
+        <v>iEcolC_1368.xml</v>
+      </c>
+      <c r="H49" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A49,".modelspec"),_xlfn.CONCAT(A49,".modelspec"))</f>
+        <v>iEcolC_1368.modelspec</v>
+      </c>
+      <c r="I49" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A49,".py"),_xlfn.CONCAT(A49,".py"))</f>
+        <v>iEcolC_1368.py</v>
+      </c>
+      <c r="J49" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEcolC_1368.py</v>
+      </c>
+      <c r="K49" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iEcolC_1368.modelspec</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A50" s="4" t="s">
         <v>88</v>
       </c>
@@ -2115,8 +3094,28 @@
       <c r="F50" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G50" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECP_1309.xml</v>
+      </c>
+      <c r="H50" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECP_1309.modelspec</v>
+      </c>
+      <c r="I50" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECP_1309.py</v>
+      </c>
+      <c r="J50" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECP_1309.py</v>
+      </c>
+      <c r="K50" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iECP_1309.modelspec</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A51" s="4" t="s">
         <v>90</v>
       </c>
@@ -2135,8 +3134,27 @@
       <c r="F51" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G51" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECs_1301.xml</v>
+      </c>
+      <c r="H51" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A51,".modelspec"),_xlfn.CONCAT(A51,".modelspec"))</f>
+        <v>iECs_1301.modelspec</v>
+      </c>
+      <c r="I51" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECs_1301.py</v>
+      </c>
+      <c r="J51" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECs_1301.py</v>
+      </c>
+      <c r="K51" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A52" s="4" t="s">
         <v>92</v>
       </c>
@@ -2155,8 +3173,27 @@
       <c r="F52" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G52" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECS88_1305.xml</v>
+      </c>
+      <c r="H52" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECS88_1305.modelspec</v>
+      </c>
+      <c r="I52" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECS88_1305.py</v>
+      </c>
+      <c r="J52" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECS88_1305.py</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A53" s="4" t="s">
         <v>94</v>
       </c>
@@ -2175,8 +3212,27 @@
       <c r="F53" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G53" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECSE_1348.xml</v>
+      </c>
+      <c r="H53" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iECSE_1348.modelspec</v>
+      </c>
+      <c r="I53" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECSE_1348.py</v>
+      </c>
+      <c r="J53" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECSE_1348.py</v>
+      </c>
+      <c r="K53" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A54" s="4" t="s">
         <v>96</v>
       </c>
@@ -2195,8 +3251,27 @@
       <c r="F54" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G54" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECSF_1327.xml</v>
+      </c>
+      <c r="H54" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A54,".modelspec"),_xlfn.CONCAT(A54,".modelspec"))</f>
+        <v>iECSF_1327.modelspec</v>
+      </c>
+      <c r="I54" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A54,".py"),_xlfn.CONCAT(A54,".py"))</f>
+        <v>iECSF_1327.py</v>
+      </c>
+      <c r="J54" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECSF_1327.py</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A55" s="4" t="s">
         <v>98</v>
       </c>
@@ -2215,8 +3290,27 @@
       <c r="F55" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G55" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A55,".xml"),_xlfn.CONCAT(A55,".xml"))</f>
+        <v>iEcSMS35_1347.xml</v>
+      </c>
+      <c r="H55" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iEcSMS35_1347.modelspec</v>
+      </c>
+      <c r="I55" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A55,".py"),_xlfn.CONCAT(A55,".py"))</f>
+        <v>iEcSMS35_1347.py</v>
+      </c>
+      <c r="J55" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEcSMS35_1347.py</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
         <v>100</v>
       </c>
@@ -2235,8 +3329,27 @@
       <c r="F56" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G56" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECSP_1301.xml</v>
+      </c>
+      <c r="H56" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A56,".modelspec"),_xlfn.CONCAT(A56,".modelspec"))</f>
+        <v>iECSP_1301.modelspec</v>
+      </c>
+      <c r="I56" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A56,".py"),_xlfn.CONCAT(A56,".py"))</f>
+        <v>iECSP_1301.py</v>
+      </c>
+      <c r="J56" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECSP_1301.py</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A57" s="4" t="s">
         <v>102</v>
       </c>
@@ -2255,8 +3368,27 @@
       <c r="F57" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G57" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECUMN_1333.xml</v>
+      </c>
+      <c r="H57" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A57,".modelspec"),_xlfn.CONCAT(A57,".modelspec"))</f>
+        <v>iECUMN_1333.modelspec</v>
+      </c>
+      <c r="I57" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECUMN_1333.py</v>
+      </c>
+      <c r="J57" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A57,".py"),_xlfn.CONCAT(A57,".py"))</f>
+        <v>iECUMN_1333.py</v>
+      </c>
+      <c r="K57" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A58" s="4" t="s">
         <v>104</v>
       </c>
@@ -2275,8 +3407,27 @@
       <c r="F58" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G58" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iECW_1372.xml</v>
+      </c>
+      <c r="H58" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A58,".modelspec"),_xlfn.CONCAT(A58,".modelspec"))</f>
+        <v>iECW_1372.modelspec</v>
+      </c>
+      <c r="I58" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iECW_1372.py</v>
+      </c>
+      <c r="J58" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iECW_1372.py</v>
+      </c>
+      <c r="K58" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A59" s="4" t="s">
         <v>105</v>
       </c>
@@ -2295,8 +3446,27 @@
       <c r="F59" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G59" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iEK1008.xml</v>
+      </c>
+      <c r="H59" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A59,".modelspec"),_xlfn.CONCAT(A59,".modelspec"))</f>
+        <v>iEK1008.modelspec</v>
+      </c>
+      <c r="I59" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iEK1008.py</v>
+      </c>
+      <c r="J59" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEK1008.py</v>
+      </c>
+      <c r="K59" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A60" s="4" t="s">
         <v>107</v>
       </c>
@@ -2315,8 +3485,27 @@
       <c r="F60" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G60" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iEKO11_1354.xml</v>
+      </c>
+      <c r="H60" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iEKO11_1354.modelspec</v>
+      </c>
+      <c r="I60" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iEKO11_1354.py</v>
+      </c>
+      <c r="J60" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iEKO11_1354.py</v>
+      </c>
+      <c r="K60" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
         <v>109</v>
       </c>
@@ -2335,8 +3524,27 @@
       <c r="F61" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G61" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iETEC_1333.xml</v>
+      </c>
+      <c r="H61" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iETEC_1333.modelspec</v>
+      </c>
+      <c r="I61" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A61,".py"),_xlfn.CONCAT(A61,".py"))</f>
+        <v>iETEC_1333.py</v>
+      </c>
+      <c r="J61" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iETEC_1333.py</v>
+      </c>
+      <c r="K61" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A62" s="4" t="s">
         <v>111</v>
       </c>
@@ -2355,8 +3563,27 @@
       <c r="F62" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G62" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iG2583_1286.xml</v>
+      </c>
+      <c r="H62" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iG2583_1286.modelspec</v>
+      </c>
+      <c r="I62" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iG2583_1286.py</v>
+      </c>
+      <c r="J62" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iG2583_1286.py</v>
+      </c>
+      <c r="K62" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A63" s="4" t="s">
         <v>113</v>
       </c>
@@ -2375,8 +3602,27 @@
       <c r="F63" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G63" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iHN637.xml</v>
+      </c>
+      <c r="H63" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iHN637.modelspec</v>
+      </c>
+      <c r="I63" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iHN637.py</v>
+      </c>
+      <c r="J63" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iHN637.py</v>
+      </c>
+      <c r="K63" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A64" s="4" t="s">
         <v>115</v>
       </c>
@@ -2395,8 +3641,27 @@
       <c r="F64" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G64" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iIS312.xml</v>
+      </c>
+      <c r="H64" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iIS312.modelspec</v>
+      </c>
+      <c r="I64" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iIS312.py</v>
+      </c>
+      <c r="J64" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iIS312.py</v>
+      </c>
+      <c r="K64" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A65" s="4" t="s">
         <v>117</v>
       </c>
@@ -2415,8 +3680,27 @@
       <c r="F65" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G65" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iIS312_Amastigote.xml</v>
+      </c>
+      <c r="H65" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A65,".modelspec"),_xlfn.CONCAT(A65,".modelspec"))</f>
+        <v>iIS312_Amastigote.modelspec</v>
+      </c>
+      <c r="I65" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iIS312_Amastigote.py</v>
+      </c>
+      <c r="J65" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iIS312_Amastigote.py</v>
+      </c>
+      <c r="K65" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A66" s="4" t="s">
         <v>118</v>
       </c>
@@ -2435,8 +3719,27 @@
       <c r="F66" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G66" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v>iIS312_Epimastigote.xml</v>
+      </c>
+      <c r="H66" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v>iIS312_Epimastigote.modelspec</v>
+      </c>
+      <c r="I66" s="14" t="str">
+        <f t="shared" si="2"/>
+        <v>iIS312_Epimastigote.py</v>
+      </c>
+      <c r="J66" s="14" t="str">
+        <f t="shared" si="3"/>
+        <v>iIS312_Epimastigote.py</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A67" s="4" t="s">
         <v>119</v>
       </c>
@@ -2455,8 +3758,27 @@
       <c r="F67" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G67" s="14" t="str">
+        <f t="shared" ref="G67:G109" si="5">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A67,".xml"),_xlfn.CONCAT(A67,".xml"))</f>
+        <v>iIS312_Trypomastigote.xml</v>
+      </c>
+      <c r="H67" s="14" t="str">
+        <f t="shared" ref="H67:H109" si="6">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A67,".modelspec"),_xlfn.CONCAT(A67,".modelspec"))</f>
+        <v>iIS312_Trypomastigote.modelspec</v>
+      </c>
+      <c r="I67" s="14" t="str">
+        <f t="shared" ref="I67:I109" si="7">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A67,".py"),_xlfn.CONCAT(A67,".py"))</f>
+        <v>iIS312_Trypomastigote.py</v>
+      </c>
+      <c r="J67" s="14" t="str">
+        <f t="shared" ref="J67:J109" si="8">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A67,".py"),_xlfn.CONCAT(A67,".py"))</f>
+        <v>iIS312_Trypomastigote.py</v>
+      </c>
+      <c r="K67" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A68" s="4" t="s">
         <v>120</v>
       </c>
@@ -2475,8 +3797,27 @@
       <c r="F68" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G68" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A68,".xml"),_xlfn.CONCAT(A68,".xml"))</f>
+        <v>iIT341.xml</v>
+      </c>
+      <c r="H68" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iIT341.modelspec</v>
+      </c>
+      <c r="I68" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iIT341.py</v>
+      </c>
+      <c r="J68" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iIT341.py</v>
+      </c>
+      <c r="K68" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A69" s="4" t="s">
         <v>122</v>
       </c>
@@ -2495,8 +3836,27 @@
       <c r="F69" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G69" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iJB785.xml</v>
+      </c>
+      <c r="H69" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iJB785.modelspec</v>
+      </c>
+      <c r="I69" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iJB785.py</v>
+      </c>
+      <c r="J69" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iJB785.py</v>
+      </c>
+      <c r="K69" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A70" s="4" t="s">
         <v>124</v>
       </c>
@@ -2515,8 +3875,27 @@
       <c r="F70" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G70" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iJN1463.xml</v>
+      </c>
+      <c r="H70" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A70,".modelspec"),_xlfn.CONCAT(A70,".modelspec"))</f>
+        <v>iJN1463.modelspec</v>
+      </c>
+      <c r="I70" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iJN1463.py</v>
+      </c>
+      <c r="J70" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iJN1463.py</v>
+      </c>
+      <c r="K70" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A71" s="4" t="s">
         <v>126</v>
       </c>
@@ -2535,8 +3914,27 @@
       <c r="F71" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G71" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iJN678.xml</v>
+      </c>
+      <c r="H71" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iJN678.modelspec</v>
+      </c>
+      <c r="I71" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iJN678.py</v>
+      </c>
+      <c r="J71" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A71,".py"),_xlfn.CONCAT(A71,".py"))</f>
+        <v>iJN678.py</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A72" s="4" t="s">
         <v>128</v>
       </c>
@@ -2555,8 +3953,27 @@
       <c r="F72" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G72" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iJN746.xml</v>
+      </c>
+      <c r="H72" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A72,".modelspec"),_xlfn.CONCAT(A72,".modelspec"))</f>
+        <v>iJN746.modelspec</v>
+      </c>
+      <c r="I72" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iJN746.py</v>
+      </c>
+      <c r="J72" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iJN746.py</v>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A73" s="4" t="s">
         <v>129</v>
       </c>
@@ -2575,8 +3992,27 @@
       <c r="F73" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G73" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iJO1366.xml</v>
+      </c>
+      <c r="H73" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iJO1366.modelspec</v>
+      </c>
+      <c r="I73" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iJO1366.py</v>
+      </c>
+      <c r="J73" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iJO1366.py</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A74" s="4" t="s">
         <v>130</v>
       </c>
@@ -2595,8 +4031,27 @@
       <c r="F74" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G74" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iJR904.xml</v>
+      </c>
+      <c r="H74" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A74,".modelspec"),_xlfn.CONCAT(A74,".modelspec"))</f>
+        <v>iJR904.modelspec</v>
+      </c>
+      <c r="I74" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iJR904.py</v>
+      </c>
+      <c r="J74" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iJR904.py</v>
+      </c>
+      <c r="K74" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A75" s="4" t="s">
         <v>131</v>
       </c>
@@ -2615,8 +4070,27 @@
       <c r="F75" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G75" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iLB1027_lipid.xml</v>
+      </c>
+      <c r="H75" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A75,".modelspec"),_xlfn.CONCAT(A75,".modelspec"))</f>
+        <v>iLB1027_lipid.modelspec</v>
+      </c>
+      <c r="I75" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A75,".py"),_xlfn.CONCAT(A75,".py"))</f>
+        <v>iLB1027_lipid.py</v>
+      </c>
+      <c r="J75" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iLB1027_lipid.py</v>
+      </c>
+      <c r="K75" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A76" s="4" t="s">
         <v>133</v>
       </c>
@@ -2635,8 +4109,27 @@
       <c r="F76" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G76" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iLF82_1304.xml</v>
+      </c>
+      <c r="H76" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iLF82_1304.modelspec</v>
+      </c>
+      <c r="I76" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iLF82_1304.py</v>
+      </c>
+      <c r="J76" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iLF82_1304.py</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A77" s="4" t="s">
         <v>135</v>
       </c>
@@ -2655,8 +4148,27 @@
       <c r="F77" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G77" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iLJ478.xml</v>
+      </c>
+      <c r="H77" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iLJ478.modelspec</v>
+      </c>
+      <c r="I77" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iLJ478.py</v>
+      </c>
+      <c r="J77" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iLJ478.py</v>
+      </c>
+      <c r="K77" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A78" s="4" t="s">
         <v>137</v>
       </c>
@@ -2675,8 +4187,27 @@
       <c r="F78" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G78" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iML1515.xml</v>
+      </c>
+      <c r="H78" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iML1515.modelspec</v>
+      </c>
+      <c r="I78" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iML1515.py</v>
+      </c>
+      <c r="J78" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iML1515.py</v>
+      </c>
+      <c r="K78" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A79" s="4" t="s">
         <v>138</v>
       </c>
@@ -2695,8 +4226,27 @@
       <c r="F79" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G79" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iMM1415.xml</v>
+      </c>
+      <c r="H79" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iMM1415.modelspec</v>
+      </c>
+      <c r="I79" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iMM1415.py</v>
+      </c>
+      <c r="J79" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iMM1415.py</v>
+      </c>
+      <c r="K79" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A80" s="4" t="s">
         <v>140</v>
       </c>
@@ -2715,8 +4265,27 @@
       <c r="F80" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G80" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iMM904.xml</v>
+      </c>
+      <c r="H80" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A80,".modelspec"),_xlfn.CONCAT(A80,".modelspec"))</f>
+        <v>iMM904.modelspec</v>
+      </c>
+      <c r="I80" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iMM904.py</v>
+      </c>
+      <c r="J80" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iMM904.py</v>
+      </c>
+      <c r="K80" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A81" s="4" t="s">
         <v>142</v>
       </c>
@@ -2735,8 +4304,27 @@
       <c r="F81" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G81" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iND750.xml</v>
+      </c>
+      <c r="H81" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iND750.modelspec</v>
+      </c>
+      <c r="I81" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iND750.py</v>
+      </c>
+      <c r="J81" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iND750.py</v>
+      </c>
+      <c r="K81" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A82" s="4" t="s">
         <v>143</v>
       </c>
@@ -2755,8 +4343,27 @@
       <c r="F82" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G82" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iNF517.xml</v>
+      </c>
+      <c r="H82" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iNF517.modelspec</v>
+      </c>
+      <c r="I82" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iNF517.py</v>
+      </c>
+      <c r="J82" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iNF517.py</v>
+      </c>
+      <c r="K82" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A83" s="4" t="s">
         <v>145</v>
       </c>
@@ -2775,8 +4382,27 @@
       <c r="F83" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G83" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iNJ661.xml</v>
+      </c>
+      <c r="H83" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A83,".modelspec"),_xlfn.CONCAT(A83,".modelspec"))</f>
+        <v>iNJ661.modelspec</v>
+      </c>
+      <c r="I83" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iNJ661.py</v>
+      </c>
+      <c r="J83" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iNJ661.py</v>
+      </c>
+      <c r="K83" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A84" s="4" t="s">
         <v>146</v>
       </c>
@@ -2795,8 +4421,27 @@
       <c r="F84" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G84" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iNRG857_1313.xml</v>
+      </c>
+      <c r="H84" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iNRG857_1313.modelspec</v>
+      </c>
+      <c r="I84" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iNRG857_1313.py</v>
+      </c>
+      <c r="J84" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iNRG857_1313.py</v>
+      </c>
+      <c r="K84" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A85" s="4" t="s">
         <v>148</v>
       </c>
@@ -2815,8 +4460,27 @@
       <c r="F85" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G85" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iPC815.xml</v>
+      </c>
+      <c r="H85" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iPC815.modelspec</v>
+      </c>
+      <c r="I85" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iPC815.py</v>
+      </c>
+      <c r="J85" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iPC815.py</v>
+      </c>
+      <c r="K85" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A86" s="4" t="s">
         <v>150</v>
       </c>
@@ -2835,8 +4499,27 @@
       <c r="F86" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G86" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iRC1080.xml</v>
+      </c>
+      <c r="H86" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A86,".modelspec"),_xlfn.CONCAT(A86,".modelspec"))</f>
+        <v>iRC1080.modelspec</v>
+      </c>
+      <c r="I86" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iRC1080.py</v>
+      </c>
+      <c r="J86" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iRC1080.py</v>
+      </c>
+      <c r="K86" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A87" s="4" t="s">
         <v>152</v>
       </c>
@@ -2855,8 +4538,27 @@
       <c r="F87" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G87" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A87,".xml"),_xlfn.CONCAT(A87,".xml"))</f>
+        <v>iS_1188.xml</v>
+      </c>
+      <c r="H87" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A87,".modelspec"),_xlfn.CONCAT(A87,".modelspec"))</f>
+        <v>iS_1188.modelspec</v>
+      </c>
+      <c r="I87" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iS_1188.py</v>
+      </c>
+      <c r="J87" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iS_1188.py</v>
+      </c>
+      <c r="K87" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A88" s="4" t="s">
         <v>154</v>
       </c>
@@ -2875,8 +4577,27 @@
       <c r="F88" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G88" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A88,".xml"),_xlfn.CONCAT(A88,".xml"))</f>
+        <v>iSB619.xml</v>
+      </c>
+      <c r="H88" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iSB619.modelspec</v>
+      </c>
+      <c r="I88" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iSB619.py</v>
+      </c>
+      <c r="J88" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iSB619.py</v>
+      </c>
+      <c r="K88" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A89" s="4" t="s">
         <v>156</v>
       </c>
@@ -2895,8 +4616,27 @@
       <c r="F89" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G89" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iSbBS512_1146.xml</v>
+      </c>
+      <c r="H89" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iSbBS512_1146.modelspec</v>
+      </c>
+      <c r="I89" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iSbBS512_1146.py</v>
+      </c>
+      <c r="J89" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iSbBS512_1146.py</v>
+      </c>
+      <c r="K89" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A90" s="4" t="s">
         <v>158</v>
       </c>
@@ -2915,8 +4655,27 @@
       <c r="F90" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G90" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iSBO_1134.xml</v>
+      </c>
+      <c r="H90" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iSBO_1134.modelspec</v>
+      </c>
+      <c r="I90" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iSBO_1134.py</v>
+      </c>
+      <c r="J90" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iSBO_1134.py</v>
+      </c>
+      <c r="K90" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A91" s="4" t="s">
         <v>160</v>
       </c>
@@ -2935,8 +4694,27 @@
       <c r="F91" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G91" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iSDY_1059.xml</v>
+      </c>
+      <c r="H91" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iSDY_1059.modelspec</v>
+      </c>
+      <c r="I91" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iSDY_1059.py</v>
+      </c>
+      <c r="J91" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iSDY_1059.py</v>
+      </c>
+      <c r="K91" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A92" s="4" t="s">
         <v>162</v>
       </c>
@@ -2955,8 +4733,27 @@
       <c r="F92" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G92" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iSF_1195.xml</v>
+      </c>
+      <c r="H92" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iSF_1195.modelspec</v>
+      </c>
+      <c r="I92" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A92,".py"),_xlfn.CONCAT(A92,".py"))</f>
+        <v>iSF_1195.py</v>
+      </c>
+      <c r="J92" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iSF_1195.py</v>
+      </c>
+      <c r="K92" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A93" s="4" t="s">
         <v>164</v>
       </c>
@@ -2975,8 +4772,27 @@
       <c r="F93" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G93" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iSFV_1184.xml</v>
+      </c>
+      <c r="H93" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iSFV_1184.modelspec</v>
+      </c>
+      <c r="I93" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iSFV_1184.py</v>
+      </c>
+      <c r="J93" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iSFV_1184.py</v>
+      </c>
+      <c r="K93" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A94" s="4" t="s">
         <v>166</v>
       </c>
@@ -2995,8 +4811,27 @@
       <c r="F94" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G94" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iSFxv_1172.xml</v>
+      </c>
+      <c r="H94" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iSFxv_1172.modelspec</v>
+      </c>
+      <c r="I94" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A94,".py"),_xlfn.CONCAT(A94,".py"))</f>
+        <v>iSFxv_1172.py</v>
+      </c>
+      <c r="J94" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iSFxv_1172.py</v>
+      </c>
+      <c r="K94" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A95" s="4" t="s">
         <v>168</v>
       </c>
@@ -3015,8 +4850,27 @@
       <c r="F95" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G95" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iSSON_1240.xml</v>
+      </c>
+      <c r="H95" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A95,".modelspec"),_xlfn.CONCAT(A95,".modelspec"))</f>
+        <v>iSSON_1240.modelspec</v>
+      </c>
+      <c r="I95" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iSSON_1240.py</v>
+      </c>
+      <c r="J95" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iSSON_1240.py</v>
+      </c>
+      <c r="K95" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A96" s="4" t="s">
         <v>170</v>
       </c>
@@ -3035,8 +4889,27 @@
       <c r="F96" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G96" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iSynCJ816.xml</v>
+      </c>
+      <c r="H96" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iSynCJ816.modelspec</v>
+      </c>
+      <c r="I96" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iSynCJ816.py</v>
+      </c>
+      <c r="J96" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iSynCJ816.py</v>
+      </c>
+      <c r="K96" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A97" s="4" t="s">
         <v>171</v>
       </c>
@@ -3055,8 +4928,27 @@
       <c r="F97" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G97" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iUMN146_1321.xml</v>
+      </c>
+      <c r="H97" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A97,".modelspec"),_xlfn.CONCAT(A97,".modelspec"))</f>
+        <v>iUMN146_1321.modelspec</v>
+      </c>
+      <c r="I97" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iUMN146_1321.py</v>
+      </c>
+      <c r="J97" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iUMN146_1321.py</v>
+      </c>
+      <c r="K97" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A98" s="4" t="s">
         <v>173</v>
       </c>
@@ -3075,8 +4967,27 @@
       <c r="F98" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G98" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iUMNK88_1353.xml</v>
+      </c>
+      <c r="H98" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iUMNK88_1353.modelspec</v>
+      </c>
+      <c r="I98" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iUMNK88_1353.py</v>
+      </c>
+      <c r="J98" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iUMNK88_1353.py</v>
+      </c>
+      <c r="K98" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A99" s="4" t="s">
         <v>175</v>
       </c>
@@ -3095,8 +5006,27 @@
       <c r="F99" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G99" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iUTI89_1310.xml</v>
+      </c>
+      <c r="H99" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iUTI89_1310.modelspec</v>
+      </c>
+      <c r="I99" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iUTI89_1310.py</v>
+      </c>
+      <c r="J99" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iUTI89_1310.py</v>
+      </c>
+      <c r="K99" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A100" s="4" t="s">
         <v>177</v>
       </c>
@@ -3115,8 +5045,27 @@
       <c r="F100" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G100" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iWFL_1372.xml</v>
+      </c>
+      <c r="H100" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iWFL_1372.modelspec</v>
+      </c>
+      <c r="I100" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iWFL_1372.py</v>
+      </c>
+      <c r="J100" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A100,".py"),_xlfn.CONCAT(A100,".py"))</f>
+        <v>iWFL_1372.py</v>
+      </c>
+      <c r="K100" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A101" s="4" t="s">
         <v>178</v>
       </c>
@@ -3135,8 +5084,27 @@
       <c r="F101" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G101" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A101,".xml"),_xlfn.CONCAT(A101,".xml"))</f>
+        <v>iY75_1357.xml</v>
+      </c>
+      <c r="H101" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iY75_1357.modelspec</v>
+      </c>
+      <c r="I101" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iY75_1357.py</v>
+      </c>
+      <c r="J101" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iY75_1357.py</v>
+      </c>
+      <c r="K101" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" ht="32" x14ac:dyDescent="0.4">
       <c r="A102" s="4" t="s">
         <v>179</v>
       </c>
@@ -3155,8 +5123,27 @@
       <c r="F102" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G102" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iYL1228.xml</v>
+      </c>
+      <c r="H102" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iYL1228.modelspec</v>
+      </c>
+      <c r="I102" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iYL1228.py</v>
+      </c>
+      <c r="J102" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iYL1228.py</v>
+      </c>
+      <c r="K102" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A103" s="4" t="s">
         <v>181</v>
       </c>
@@ -3175,8 +5162,27 @@
       <c r="F103" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G103" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A103,".xml"),_xlfn.CONCAT(A103,".xml"))</f>
+        <v>iYO844.xml</v>
+      </c>
+      <c r="H103" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iYO844.modelspec</v>
+      </c>
+      <c r="I103" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iYO844.py</v>
+      </c>
+      <c r="J103" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A103,".py"),_xlfn.CONCAT(A103,".py"))</f>
+        <v>iYO844.py</v>
+      </c>
+      <c r="K103" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A104" s="4" t="s">
         <v>183</v>
       </c>
@@ -3195,8 +5201,27 @@
       <c r="F104" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G104" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iYS1720.xml</v>
+      </c>
+      <c r="H104" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iYS1720.modelspec</v>
+      </c>
+      <c r="I104" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iYS1720.py</v>
+      </c>
+      <c r="J104" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iYS1720.py</v>
+      </c>
+      <c r="K104" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" ht="32" x14ac:dyDescent="0.4">
       <c r="A105" s="4" t="s">
         <v>185</v>
       </c>
@@ -3215,8 +5240,27 @@
       <c r="F105" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G105" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iYS854.xml</v>
+      </c>
+      <c r="H105" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A105,".modelspec"),_xlfn.CONCAT(A105,".modelspec"))</f>
+        <v>iYS854.modelspec</v>
+      </c>
+      <c r="I105" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iYS854.py</v>
+      </c>
+      <c r="J105" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iYS854.py</v>
+      </c>
+      <c r="K105" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A106" s="4" t="s">
         <v>187</v>
       </c>
@@ -3235,8 +5279,27 @@
       <c r="F106" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G106" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>iZ_1308.xml</v>
+      </c>
+      <c r="H106" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>iZ_1308.modelspec</v>
+      </c>
+      <c r="I106" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>iZ_1308.py</v>
+      </c>
+      <c r="J106" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>iZ_1308.py</v>
+      </c>
+      <c r="K106" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A107" s="4" t="s">
         <v>189</v>
       </c>
@@ -3255,8 +5318,27 @@
       <c r="F107" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G107" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>RECON1.xml</v>
+      </c>
+      <c r="H107" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A107,".modelspec"),_xlfn.CONCAT(A107,".modelspec"))</f>
+        <v>RECON1.modelspec</v>
+      </c>
+      <c r="I107" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>RECON1.py</v>
+      </c>
+      <c r="J107" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>RECON1.py</v>
+      </c>
+      <c r="K107" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A108" s="4" t="s">
         <v>190</v>
       </c>
@@ -3275,8 +5357,27 @@
       <c r="F108" s="7" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="G108" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>Recon3D.xml</v>
+      </c>
+      <c r="H108" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>Recon3D.modelspec</v>
+      </c>
+      <c r="I108" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>Recon3D.py</v>
+      </c>
+      <c r="J108" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>Recon3D.py</v>
+      </c>
+      <c r="K108" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" ht="32" x14ac:dyDescent="0.4">
       <c r="A109" s="4" t="s">
         <v>191</v>
       </c>
@@ -3294,6 +5395,25 @@
       </c>
       <c r="F109" s="7" t="s">
         <v>199</v>
+      </c>
+      <c r="G109" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v>STM_v1_0.xml</v>
+      </c>
+      <c r="H109" s="14" t="str">
+        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A109,".modelspec"),_xlfn.CONCAT(A109,".modelspec"))</f>
+        <v>STM_v1_0.modelspec</v>
+      </c>
+      <c r="I109" s="14" t="str">
+        <f t="shared" si="7"/>
+        <v>STM_v1_0.py</v>
+      </c>
+      <c r="J109" s="14" t="str">
+        <f t="shared" si="8"/>
+        <v>STM_v1_0.py</v>
+      </c>
+      <c r="K109" s="1" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
# updated list of GSM converted KMs
</commit_message>
<xml_diff>
--- a/List of GSM-Converted Kinetic Models.xlsx
+++ b/List of GSM-Converted Kinetic Models.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\MyProjects\kinmodre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB75B7FC-5D93-43E8-B30D-8EBB33DB801D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B8BB40-C43D-462A-92FB-85E52B809379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B4C7D942-9A2E-4284-ADB5-B7C4CF7DD1B1}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="206">
   <si>
     <t>e_coli_core</t>
   </si>
@@ -655,9 +655,6 @@
   </si>
   <si>
     <t>ODE Script File (in GSM-odescripts folder)</t>
-  </si>
-  <si>
-    <t>OK</t>
   </si>
 </sst>
 </file>
@@ -748,7 +745,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -784,9 +781,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
@@ -1127,13 +1121,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC6CDDD6-2BE3-467B-8E7F-78A96156F001}">
-  <dimension ref="A1:K109"/>
+  <dimension ref="A1:J109"/>
   <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22.81640625" style="7" customWidth="1"/>
     <col min="2" max="2" width="40" style="7" customWidth="1"/>
-    <col min="3" max="5" width="14" style="8" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="10.26953125" style="7" hidden="1" customWidth="1"/>
+    <col min="3" max="5" width="14" style="8" customWidth="1"/>
+    <col min="6" max="6" width="10.26953125" style="7" customWidth="1"/>
     <col min="7" max="7" width="21.6328125" style="7" customWidth="1"/>
     <col min="8" max="8" width="24.90625" style="7" customWidth="1"/>
     <col min="9" max="10" width="21.6328125" style="7" customWidth="1"/>
@@ -1142,7 +1136,7 @@
     <col min="13" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>193</v>
       </c>
@@ -1174,7 +1168,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1193,27 +1187,24 @@
       <c r="F2" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G2" s="14" t="str">
+      <c r="G2" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A2,".xml"),_xlfn.CONCAT(A2,".xml"))</f>
         <v>e_coli_core.xml</v>
       </c>
-      <c r="H2" s="14" t="str">
+      <c r="H2" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A2,".modelspec"),_xlfn.CONCAT(A2,".modelspec"))</f>
         <v>e_coli_core.modelspec</v>
       </c>
-      <c r="I2" s="14" t="str">
+      <c r="I2" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A2,".py"),_xlfn.CONCAT(A2,".py"))</f>
         <v>e_coli_core.py</v>
       </c>
-      <c r="J2" s="14" t="str">
+      <c r="J2" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A2,".py"),_xlfn.CONCAT(A2,".py"))</f>
         <v>e_coli_core.py</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1232,27 +1223,24 @@
       <c r="F3" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G3" s="14" t="str">
+      <c r="G3" s="13" t="str">
         <f t="shared" ref="G3:G66" si="0">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A3,".xml"),_xlfn.CONCAT(A3,".xml"))</f>
         <v>iAB_RBC_283.xml</v>
       </c>
-      <c r="H3" s="14" t="str">
+      <c r="H3" s="13" t="str">
         <f t="shared" ref="H3:H66" si="1">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A3,".modelspec"),_xlfn.CONCAT(A3,".modelspec"))</f>
         <v>iAB_RBC_283.modelspec</v>
       </c>
-      <c r="I3" s="14" t="str">
+      <c r="I3" s="13" t="str">
         <f t="shared" ref="I3:I66" si="2">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A3,".py"),_xlfn.CONCAT(A3,".py"))</f>
         <v>iAB_RBC_283.py</v>
       </c>
-      <c r="J3" s="14" t="str">
+      <c r="J3" s="13" t="str">
         <f t="shared" ref="J3:J66" si="3">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A3,".py"),_xlfn.CONCAT(A3,".py"))</f>
         <v>iAB_RBC_283.py</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -1271,27 +1259,24 @@
       <c r="F4" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G4" s="14" t="str">
+      <c r="G4" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iAF1260.xml</v>
       </c>
-      <c r="H4" s="14" t="str">
+      <c r="H4" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iAF1260.modelspec</v>
       </c>
-      <c r="I4" s="14" t="str">
+      <c r="I4" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A4,".py"),_xlfn.CONCAT(A4,".py"))</f>
         <v>iAF1260.py</v>
       </c>
-      <c r="J4" s="14" t="str">
+      <c r="J4" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iAF1260.py</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
@@ -1310,27 +1295,24 @@
       <c r="F5" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G5" s="14" t="str">
+      <c r="G5" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iAF1260b.xml</v>
       </c>
-      <c r="H5" s="14" t="str">
+      <c r="H5" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iAF1260b.modelspec</v>
       </c>
-      <c r="I5" s="14" t="str">
+      <c r="I5" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iAF1260b.py</v>
       </c>
-      <c r="J5" s="14" t="str">
+      <c r="J5" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iAF1260b.py</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
@@ -1349,27 +1331,24 @@
       <c r="F6" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G6" s="14" t="str">
+      <c r="G6" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iAF692.xml</v>
       </c>
-      <c r="H6" s="14" t="str">
+      <c r="H6" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iAF692.modelspec</v>
       </c>
-      <c r="I6" s="14" t="str">
+      <c r="I6" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iAF692.py</v>
       </c>
-      <c r="J6" s="14" t="str">
+      <c r="J6" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iAF692.py</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
@@ -1388,27 +1367,24 @@
       <c r="F7" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G7" s="14" t="str">
+      <c r="G7" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iAF987.xml</v>
       </c>
-      <c r="H7" s="14" t="str">
+      <c r="H7" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iAF987.modelspec</v>
       </c>
-      <c r="I7" s="14" t="str">
+      <c r="I7" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iAF987.py</v>
       </c>
-      <c r="J7" s="14" t="str">
+      <c r="J7" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iAF987.py</v>
       </c>
-      <c r="K7" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
@@ -1427,27 +1403,24 @@
       <c r="F8" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G8" s="14" t="str">
+      <c r="G8" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A8,".xml"),_xlfn.CONCAT(A8,".xml"))</f>
         <v>iAM_Pb448.xml</v>
       </c>
-      <c r="H8" s="14" t="str">
+      <c r="H8" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iAM_Pb448.modelspec</v>
       </c>
-      <c r="I8" s="14" t="str">
+      <c r="I8" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iAM_Pb448.py</v>
       </c>
-      <c r="J8" s="14" t="str">
+      <c r="J8" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iAM_Pb448.py</v>
       </c>
-      <c r="K8" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
@@ -1466,27 +1439,24 @@
       <c r="F9" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G9" s="14" t="str">
+      <c r="G9" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iAM_Pc455.xml</v>
       </c>
-      <c r="H9" s="14" t="str">
+      <c r="H9" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iAM_Pc455.modelspec</v>
       </c>
-      <c r="I9" s="14" t="str">
+      <c r="I9" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A9,".py"),_xlfn.CONCAT(A9,".py"))</f>
         <v>iAM_Pc455.py</v>
       </c>
-      <c r="J9" s="14" t="str">
+      <c r="J9" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iAM_Pc455.py</v>
       </c>
-      <c r="K9" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
@@ -1505,27 +1475,24 @@
       <c r="F10" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G10" s="14" t="str">
+      <c r="G10" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iAM_Pf480.xml</v>
       </c>
-      <c r="H10" s="14" t="str">
+      <c r="H10" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iAM_Pf480.modelspec</v>
       </c>
-      <c r="I10" s="14" t="str">
+      <c r="I10" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A10,".py"),_xlfn.CONCAT(A10,".py"))</f>
         <v>iAM_Pf480.py</v>
       </c>
-      <c r="J10" s="14" t="str">
+      <c r="J10" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A10,".py"),_xlfn.CONCAT(A10,".py"))</f>
         <v>iAM_Pf480.py</v>
       </c>
-      <c r="K10" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>16</v>
       </c>
@@ -1544,27 +1511,24 @@
       <c r="F11" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G11" s="14" t="str">
+      <c r="G11" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A11,".xml"),_xlfn.CONCAT(A11,".xml"))</f>
         <v>iAM_Pk459.xml</v>
       </c>
-      <c r="H11" s="14" t="str">
+      <c r="H11" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A11,".modelspec"),_xlfn.CONCAT(A11,".modelspec"))</f>
         <v>iAM_Pk459.modelspec</v>
       </c>
-      <c r="I11" s="14" t="str">
+      <c r="I11" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iAM_Pk459.py</v>
       </c>
-      <c r="J11" s="14" t="str">
+      <c r="J11" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iAM_Pk459.py</v>
       </c>
-      <c r="K11" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>18</v>
       </c>
@@ -1583,27 +1547,24 @@
       <c r="F12" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G12" s="14" t="str">
+      <c r="G12" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iAM_Pv461.xml</v>
       </c>
-      <c r="H12" s="14" t="str">
+      <c r="H12" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iAM_Pv461.modelspec</v>
       </c>
-      <c r="I12" s="14" t="str">
+      <c r="I12" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A12,".py"),_xlfn.CONCAT(A12,".py"))</f>
         <v>iAM_Pv461.py</v>
       </c>
-      <c r="J12" s="14" t="str">
+      <c r="J12" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iAM_Pv461.py</v>
       </c>
-      <c r="K12" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>20</v>
       </c>
@@ -1622,27 +1583,24 @@
       <c r="F13" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G13" s="14" t="str">
+      <c r="G13" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iAPECO1_1312.xml</v>
       </c>
-      <c r="H13" s="14" t="str">
+      <c r="H13" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iAPECO1_1312.modelspec</v>
       </c>
-      <c r="I13" s="14" t="str">
+      <c r="I13" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A13,".py"),_xlfn.CONCAT(A13,".py"))</f>
         <v>iAPECO1_1312.py</v>
       </c>
-      <c r="J13" s="14" t="str">
+      <c r="J13" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A13,".py"),_xlfn.CONCAT(A13,".py"))</f>
         <v>iAPECO1_1312.py</v>
       </c>
-      <c r="K13" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A14" s="4" t="s">
         <v>22</v>
       </c>
@@ -1661,27 +1619,24 @@
       <c r="F14" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G14" s="14" t="str">
+      <c r="G14" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iAT_PLT_636.xml</v>
       </c>
-      <c r="H14" s="14" t="str">
+      <c r="H14" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iAT_PLT_636.modelspec</v>
       </c>
-      <c r="I14" s="14" t="str">
+      <c r="I14" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A14,".py"),_xlfn.CONCAT(A14,".py"))</f>
         <v>iAT_PLT_636.py</v>
       </c>
-      <c r="J14" s="14" t="str">
+      <c r="J14" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iAT_PLT_636.py</v>
       </c>
-      <c r="K14" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A15" s="4" t="s">
         <v>23</v>
       </c>
@@ -1700,27 +1655,24 @@
       <c r="F15" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G15" s="14" t="str">
+      <c r="G15" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iB21_1397.xml</v>
       </c>
-      <c r="H15" s="14" t="str">
+      <c r="H15" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iB21_1397.modelspec</v>
       </c>
-      <c r="I15" s="14" t="str">
+      <c r="I15" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A15,".py"),_xlfn.CONCAT(A15,".py"))</f>
         <v>iB21_1397.py</v>
       </c>
-      <c r="J15" s="14" t="str">
+      <c r="J15" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A15,".py"),_xlfn.CONCAT(A15,".py"))</f>
         <v>iB21_1397.py</v>
       </c>
-      <c r="K15" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A16" s="4" t="s">
         <v>25</v>
       </c>
@@ -1739,27 +1691,24 @@
       <c r="F16" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G16" s="14" t="str">
+      <c r="G16" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iBWG_1329.xml</v>
       </c>
-      <c r="H16" s="14" t="str">
+      <c r="H16" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iBWG_1329.modelspec</v>
       </c>
-      <c r="I16" s="14" t="str">
+      <c r="I16" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iBWG_1329.py</v>
       </c>
-      <c r="J16" s="14" t="str">
+      <c r="J16" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A16,".py"),_xlfn.CONCAT(A16,".py"))</f>
         <v>iBWG_1329.py</v>
       </c>
-      <c r="K16" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A17" s="4" t="s">
         <v>27</v>
       </c>
@@ -1778,27 +1727,24 @@
       <c r="F17" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G17" s="14" t="str">
+      <c r="G17" s="13" t="str">
         <f t="shared" si="0"/>
         <v>ic_1306.xml</v>
       </c>
-      <c r="H17" s="14" t="str">
+      <c r="H17" s="13" t="str">
         <f t="shared" si="1"/>
         <v>ic_1306.modelspec</v>
       </c>
-      <c r="I17" s="14" t="str">
+      <c r="I17" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A17,".py"),_xlfn.CONCAT(A17,".py"))</f>
         <v>ic_1306.py</v>
       </c>
-      <c r="J17" s="14" t="str">
+      <c r="J17" s="13" t="str">
         <f t="shared" si="3"/>
         <v>ic_1306.py</v>
       </c>
-      <c r="K17" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A18" s="4" t="s">
         <v>29</v>
       </c>
@@ -1817,27 +1763,24 @@
       <c r="F18" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G18" s="14" t="str">
+      <c r="G18" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A18,".xml"),_xlfn.CONCAT(A18,".xml"))</f>
         <v>iCHOv1.xml</v>
       </c>
-      <c r="H18" s="14" t="str">
+      <c r="H18" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iCHOv1.modelspec</v>
       </c>
-      <c r="I18" s="14" t="str">
+      <c r="I18" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iCHOv1.py</v>
       </c>
-      <c r="J18" s="14" t="str">
+      <c r="J18" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iCHOv1.py</v>
       </c>
-      <c r="K18" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
         <v>31</v>
       </c>
@@ -1856,28 +1799,24 @@
       <c r="F19" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G19" s="14" t="str">
+      <c r="G19" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iCHOv1_DG44.xml</v>
       </c>
-      <c r="H19" s="14" t="str">
+      <c r="H19" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A19,".modelspec"),_xlfn.CONCAT(A19,".modelspec"))</f>
         <v>iCHOv1_DG44.modelspec</v>
       </c>
-      <c r="I19" s="14" t="str">
+      <c r="I19" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iCHOv1_DG44.py</v>
       </c>
-      <c r="J19" s="14" t="str">
+      <c r="J19" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iCHOv1_DG44.py</v>
       </c>
-      <c r="K19" s="13" t="str">
-        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/Minionnick/kinmodre/tree/main/asm/",A19,".modelspec"),_xlfn.CONCAT(A19,".modelspec"))</f>
-        <v>iCHOv1_DG44.modelspec</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
@@ -1896,28 +1835,24 @@
       <c r="F20" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G20" s="14" t="str">
+      <c r="G20" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iCN718.xml</v>
       </c>
-      <c r="H20" s="14" t="str">
+      <c r="H20" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iCN718.modelspec</v>
       </c>
-      <c r="I20" s="14" t="str">
+      <c r="I20" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iCN718.py</v>
       </c>
-      <c r="J20" s="14" t="str">
+      <c r="J20" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iCN718.py</v>
       </c>
-      <c r="K20" s="13" t="str">
-        <f t="shared" ref="K20:K50" si="4">HYPERLINK(_xlfn.CONCAT("https://github.com/Minionnick/kinmodre/tree/main/asm/",A20,".modelspec"),_xlfn.CONCAT(A20,".modelspec"))</f>
-        <v>iCN718.modelspec</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A21" s="4" t="s">
         <v>34</v>
       </c>
@@ -1936,28 +1871,24 @@
       <c r="F21" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G21" s="14" t="str">
+      <c r="G21" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iCN900.xml</v>
       </c>
-      <c r="H21" s="14" t="str">
+      <c r="H21" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iCN900.modelspec</v>
       </c>
-      <c r="I21" s="14" t="str">
+      <c r="I21" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A21,".py"),_xlfn.CONCAT(A21,".py"))</f>
         <v>iCN900.py</v>
       </c>
-      <c r="J21" s="14" t="str">
+      <c r="J21" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A21,".py"),_xlfn.CONCAT(A21,".py"))</f>
         <v>iCN900.py</v>
       </c>
-      <c r="K21" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iCN900.modelspec</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
         <v>36</v>
       </c>
@@ -1976,28 +1907,24 @@
       <c r="F22" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G22" s="14" t="str">
+      <c r="G22" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iE2348C_1286.xml</v>
       </c>
-      <c r="H22" s="14" t="str">
+      <c r="H22" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iE2348C_1286.modelspec</v>
       </c>
-      <c r="I22" s="14" t="str">
+      <c r="I22" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iE2348C_1286.py</v>
       </c>
-      <c r="J22" s="14" t="str">
+      <c r="J22" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A22,".py"),_xlfn.CONCAT(A22,".py"))</f>
         <v>iE2348C_1286.py</v>
       </c>
-      <c r="K22" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iE2348C_1286.modelspec</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A23" s="4" t="s">
         <v>38</v>
       </c>
@@ -2016,28 +1943,24 @@
       <c r="F23" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G23" s="14" t="str">
+      <c r="G23" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A23,".xml"),_xlfn.CONCAT(A23,".xml"))</f>
         <v>iEC042_1314.xml</v>
       </c>
-      <c r="H23" s="14" t="str">
+      <c r="H23" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iEC042_1314.modelspec</v>
       </c>
-      <c r="I23" s="14" t="str">
+      <c r="I23" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A23,".py"),_xlfn.CONCAT(A23,".py"))</f>
         <v>iEC042_1314.py</v>
       </c>
-      <c r="J23" s="14" t="str">
+      <c r="J23" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEC042_1314.py</v>
       </c>
-      <c r="K23" s="13" t="str">
-        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/Minionnick/kinmodre/tree/main/asm/",A23,".modelspec"),_xlfn.CONCAT(A23,".modelspec"))</f>
-        <v>iEC042_1314.modelspec</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A24" s="4" t="s">
         <v>40</v>
       </c>
@@ -2056,28 +1979,24 @@
       <c r="F24" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G24" s="14" t="str">
+      <c r="G24" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A24,".xml"),_xlfn.CONCAT(A24,".xml"))</f>
         <v>iEC1344_C.xml</v>
       </c>
-      <c r="H24" s="14" t="str">
+      <c r="H24" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A24,".modelspec"),_xlfn.CONCAT(A24,".modelspec"))</f>
         <v>iEC1344_C.modelspec</v>
       </c>
-      <c r="I24" s="14" t="str">
+      <c r="I24" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iEC1344_C.py</v>
       </c>
-      <c r="J24" s="14" t="str">
+      <c r="J24" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEC1344_C.py</v>
       </c>
-      <c r="K24" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iEC1344_C.modelspec</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A25" s="4" t="s">
         <v>42</v>
       </c>
@@ -2096,28 +2015,24 @@
       <c r="F25" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G25" s="14" t="str">
+      <c r="G25" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iEC1349_Crooks.xml</v>
       </c>
-      <c r="H25" s="14" t="str">
+      <c r="H25" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iEC1349_Crooks.modelspec</v>
       </c>
-      <c r="I25" s="14" t="str">
+      <c r="I25" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iEC1349_Crooks.py</v>
       </c>
-      <c r="J25" s="14" t="str">
+      <c r="J25" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEC1349_Crooks.py</v>
       </c>
-      <c r="K25" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iEC1349_Crooks.modelspec</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
         <v>44</v>
       </c>
@@ -2136,28 +2051,24 @@
       <c r="F26" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G26" s="14" t="str">
+      <c r="G26" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iEC1356_Bl21DE3.xml</v>
       </c>
-      <c r="H26" s="14" t="str">
+      <c r="H26" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iEC1356_Bl21DE3.modelspec</v>
       </c>
-      <c r="I26" s="14" t="str">
+      <c r="I26" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iEC1356_Bl21DE3.py</v>
       </c>
-      <c r="J26" s="14" t="str">
+      <c r="J26" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A26,".py"),_xlfn.CONCAT(A26,".py"))</f>
         <v>iEC1356_Bl21DE3.py</v>
       </c>
-      <c r="K26" s="13" t="str">
-        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/Minionnick/kinmodre/tree/main/asm/",A26,".modelspec"),_xlfn.CONCAT(A26,".modelspec"))</f>
-        <v>iEC1356_Bl21DE3.modelspec</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A27" s="4" t="s">
         <v>45</v>
       </c>
@@ -2176,28 +2087,24 @@
       <c r="F27" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G27" s="14" t="str">
+      <c r="G27" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iEC1364_W.xml</v>
       </c>
-      <c r="H27" s="14" t="str">
+      <c r="H27" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A27,".modelspec"),_xlfn.CONCAT(A27,".modelspec"))</f>
         <v>iEC1364_W.modelspec</v>
       </c>
-      <c r="I27" s="14" t="str">
+      <c r="I27" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iEC1364_W.py</v>
       </c>
-      <c r="J27" s="14" t="str">
+      <c r="J27" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEC1364_W.py</v>
       </c>
-      <c r="K27" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iEC1364_W.modelspec</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
         <v>47</v>
       </c>
@@ -2216,28 +2123,24 @@
       <c r="F28" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G28" s="14" t="str">
+      <c r="G28" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iEC1368_DH5a.xml</v>
       </c>
-      <c r="H28" s="14" t="str">
+      <c r="H28" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A28,".modelspec"),_xlfn.CONCAT(A28,".modelspec"))</f>
         <v>iEC1368_DH5a.modelspec</v>
       </c>
-      <c r="I28" s="14" t="str">
+      <c r="I28" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iEC1368_DH5a.py</v>
       </c>
-      <c r="J28" s="14" t="str">
+      <c r="J28" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A28,".py"),_xlfn.CONCAT(A28,".py"))</f>
         <v>iEC1368_DH5a.py</v>
       </c>
-      <c r="K28" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iEC1368_DH5a.modelspec</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
         <v>49</v>
       </c>
@@ -2256,28 +2159,24 @@
       <c r="F29" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G29" s="14" t="str">
+      <c r="G29" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iEC1372_W3110.xml</v>
       </c>
-      <c r="H29" s="14" t="str">
+      <c r="H29" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iEC1372_W3110.modelspec</v>
       </c>
-      <c r="I29" s="14" t="str">
+      <c r="I29" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iEC1372_W3110.py</v>
       </c>
-      <c r="J29" s="14" t="str">
+      <c r="J29" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEC1372_W3110.py</v>
       </c>
-      <c r="K29" s="13" t="str">
-        <f>HYPERLINK(_xlfn.CONCAT("https://github.com/Minionnick/kinmodre/tree/main/asm/",A29,".modelspec"),_xlfn.CONCAT(A29,".modelspec"))</f>
-        <v>iEC1372_W3110.modelspec</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A30" s="4" t="s">
         <v>51</v>
       </c>
@@ -2296,28 +2195,24 @@
       <c r="F30" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G30" s="14" t="str">
+      <c r="G30" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iEC55989_1330.xml</v>
       </c>
-      <c r="H30" s="14" t="str">
+      <c r="H30" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iEC55989_1330.modelspec</v>
       </c>
-      <c r="I30" s="14" t="str">
+      <c r="I30" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iEC55989_1330.py</v>
       </c>
-      <c r="J30" s="14" t="str">
+      <c r="J30" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEC55989_1330.py</v>
       </c>
-      <c r="K30" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iEC55989_1330.modelspec</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A31" s="4" t="s">
         <v>53</v>
       </c>
@@ -2336,28 +2231,24 @@
       <c r="F31" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G31" s="14" t="str">
+      <c r="G31" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A31,".xml"),_xlfn.CONCAT(A31,".xml"))</f>
         <v>iECABU_c1320.xml</v>
       </c>
-      <c r="H31" s="14" t="str">
+      <c r="H31" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A31,".modelspec"),_xlfn.CONCAT(A31,".modelspec"))</f>
         <v>iECABU_c1320.modelspec</v>
       </c>
-      <c r="I31" s="14" t="str">
+      <c r="I31" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECABU_c1320.py</v>
       </c>
-      <c r="J31" s="14" t="str">
+      <c r="J31" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECABU_c1320.py</v>
       </c>
-      <c r="K31" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECABU_c1320.modelspec</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
         <v>55</v>
       </c>
@@ -2376,28 +2267,24 @@
       <c r="F32" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G32" s="14" t="str">
+      <c r="G32" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECB_1328.xml</v>
       </c>
-      <c r="H32" s="14" t="str">
+      <c r="H32" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A32,".modelspec"),_xlfn.CONCAT(A32,".modelspec"))</f>
         <v>iECB_1328.modelspec</v>
       </c>
-      <c r="I32" s="14" t="str">
+      <c r="I32" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECB_1328.py</v>
       </c>
-      <c r="J32" s="14" t="str">
+      <c r="J32" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A32,".py"),_xlfn.CONCAT(A32,".py"))</f>
         <v>iECB_1328.py</v>
       </c>
-      <c r="K32" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECB_1328.modelspec</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A33" s="4" t="s">
         <v>57</v>
       </c>
@@ -2416,28 +2303,24 @@
       <c r="F33" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G33" s="14" t="str">
+      <c r="G33" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECBD_1354.xml</v>
       </c>
-      <c r="H33" s="14" t="str">
+      <c r="H33" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECBD_1354.modelspec</v>
       </c>
-      <c r="I33" s="14" t="str">
+      <c r="I33" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECBD_1354.py</v>
       </c>
-      <c r="J33" s="14" t="str">
+      <c r="J33" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A33,".py"),_xlfn.CONCAT(A33,".py"))</f>
         <v>iECBD_1354.py</v>
       </c>
-      <c r="K33" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECBD_1354.modelspec</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A34" s="4" t="s">
         <v>59</v>
       </c>
@@ -2456,28 +2339,24 @@
       <c r="F34" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G34" s="14" t="str">
+      <c r="G34" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A34,".xml"),_xlfn.CONCAT(A34,".xml"))</f>
         <v>iECD_1391.xml</v>
       </c>
-      <c r="H34" s="14" t="str">
+      <c r="H34" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECD_1391.modelspec</v>
       </c>
-      <c r="I34" s="14" t="str">
+      <c r="I34" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A34,".py"),_xlfn.CONCAT(A34,".py"))</f>
         <v>iECD_1391.py</v>
       </c>
-      <c r="J34" s="14" t="str">
+      <c r="J34" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A34,".py"),_xlfn.CONCAT(A34,".py"))</f>
         <v>iECD_1391.py</v>
       </c>
-      <c r="K34" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECD_1391.modelspec</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A35" s="4" t="s">
         <v>60</v>
       </c>
@@ -2496,28 +2375,24 @@
       <c r="F35" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G35" s="14" t="str">
+      <c r="G35" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECDH10B_1368.xml</v>
       </c>
-      <c r="H35" s="14" t="str">
+      <c r="H35" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A35,".modelspec"),_xlfn.CONCAT(A35,".modelspec"))</f>
         <v>iECDH10B_1368.modelspec</v>
       </c>
-      <c r="I35" s="14" t="str">
+      <c r="I35" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECDH10B_1368.py</v>
       </c>
-      <c r="J35" s="14" t="str">
+      <c r="J35" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECDH10B_1368.py</v>
       </c>
-      <c r="K35" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECDH10B_1368.modelspec</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A36" s="4" t="s">
         <v>62</v>
       </c>
@@ -2536,28 +2411,24 @@
       <c r="F36" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G36" s="14" t="str">
+      <c r="G36" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iEcDH1_1363.xml</v>
       </c>
-      <c r="H36" s="14" t="str">
+      <c r="H36" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iEcDH1_1363.modelspec</v>
       </c>
-      <c r="I36" s="14" t="str">
+      <c r="I36" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A36,".py"),_xlfn.CONCAT(A36,".py"))</f>
         <v>iEcDH1_1363.py</v>
       </c>
-      <c r="J36" s="14" t="str">
+      <c r="J36" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEcDH1_1363.py</v>
       </c>
-      <c r="K36" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iEcDH1_1363.modelspec</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
+    </row>
+    <row r="37" spans="1:10" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A37" s="4" t="s">
         <v>64</v>
       </c>
@@ -2576,28 +2447,24 @@
       <c r="F37" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G37" s="14" t="str">
+      <c r="G37" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECDH1ME8569_1439.xml</v>
       </c>
-      <c r="H37" s="14" t="str">
+      <c r="H37" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECDH1ME8569_1439.modelspec</v>
       </c>
-      <c r="I37" s="14" t="str">
+      <c r="I37" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A37,".py"),_xlfn.CONCAT(A37,".py"))</f>
         <v>iECDH1ME8569_1439.py</v>
       </c>
-      <c r="J37" s="14" t="str">
+      <c r="J37" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECDH1ME8569_1439.py</v>
       </c>
-      <c r="K37" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECDH1ME8569_1439.modelspec</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A38" s="4" t="s">
         <v>65</v>
       </c>
@@ -2616,28 +2483,24 @@
       <c r="F38" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G38" s="14" t="str">
+      <c r="G38" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iEcE24377_1341.xml</v>
       </c>
-      <c r="H38" s="14" t="str">
+      <c r="H38" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iEcE24377_1341.modelspec</v>
       </c>
-      <c r="I38" s="14" t="str">
+      <c r="I38" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iEcE24377_1341.py</v>
       </c>
-      <c r="J38" s="14" t="str">
+      <c r="J38" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEcE24377_1341.py</v>
       </c>
-      <c r="K38" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iEcE24377_1341.modelspec</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A39" s="4" t="s">
         <v>67</v>
       </c>
@@ -2656,28 +2519,24 @@
       <c r="F39" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G39" s="14" t="str">
+      <c r="G39" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECED1_1282.xml</v>
       </c>
-      <c r="H39" s="14" t="str">
+      <c r="H39" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECED1_1282.modelspec</v>
       </c>
-      <c r="I39" s="14" t="str">
+      <c r="I39" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECED1_1282.py</v>
       </c>
-      <c r="J39" s="14" t="str">
+      <c r="J39" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECED1_1282.py</v>
       </c>
-      <c r="K39" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECED1_1282.modelspec</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A40" s="4" t="s">
         <v>69</v>
       </c>
@@ -2696,28 +2555,24 @@
       <c r="F40" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G40" s="14" t="str">
+      <c r="G40" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A40,".xml"),_xlfn.CONCAT(A40,".xml"))</f>
         <v>iECH74115_1262.xml</v>
       </c>
-      <c r="H40" s="14" t="str">
+      <c r="H40" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECH74115_1262.modelspec</v>
       </c>
-      <c r="I40" s="14" t="str">
+      <c r="I40" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECH74115_1262.py</v>
       </c>
-      <c r="J40" s="14" t="str">
+      <c r="J40" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECH74115_1262.py</v>
       </c>
-      <c r="K40" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECH74115_1262.modelspec</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A41" s="4" t="s">
         <v>71</v>
       </c>
@@ -2736,28 +2591,24 @@
       <c r="F41" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G41" s="14" t="str">
+      <c r="G41" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iEcHS_1320.xml</v>
       </c>
-      <c r="H41" s="14" t="str">
+      <c r="H41" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iEcHS_1320.modelspec</v>
       </c>
-      <c r="I41" s="14" t="str">
+      <c r="I41" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iEcHS_1320.py</v>
       </c>
-      <c r="J41" s="14" t="str">
+      <c r="J41" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEcHS_1320.py</v>
       </c>
-      <c r="K41" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iEcHS_1320.modelspec</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A42" s="4" t="s">
         <v>73</v>
       </c>
@@ -2776,28 +2627,24 @@
       <c r="F42" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G42" s="14" t="str">
+      <c r="G42" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A42,".xml"),_xlfn.CONCAT(A42,".xml"))</f>
         <v>iECIAI1_1343.xml</v>
       </c>
-      <c r="H42" s="14" t="str">
+      <c r="H42" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECIAI1_1343.modelspec</v>
       </c>
-      <c r="I42" s="14" t="str">
+      <c r="I42" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A42,".py"),_xlfn.CONCAT(A42,".py"))</f>
         <v>iECIAI1_1343.py</v>
       </c>
-      <c r="J42" s="14" t="str">
+      <c r="J42" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A42,".py"),_xlfn.CONCAT(A42,".py"))</f>
         <v>iECIAI1_1343.py</v>
       </c>
-      <c r="K42" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECIAI1_1343.modelspec</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A43" s="4" t="s">
         <v>75</v>
       </c>
@@ -2816,28 +2663,24 @@
       <c r="F43" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G43" s="14" t="str">
+      <c r="G43" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECIAI39_1322.xml</v>
       </c>
-      <c r="H43" s="14" t="str">
+      <c r="H43" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECIAI39_1322.modelspec</v>
       </c>
-      <c r="I43" s="14" t="str">
+      <c r="I43" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECIAI39_1322.py</v>
       </c>
-      <c r="J43" s="14" t="str">
+      <c r="J43" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECIAI39_1322.py</v>
       </c>
-      <c r="K43" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECIAI39_1322.modelspec</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A44" s="4" t="s">
         <v>77</v>
       </c>
@@ -2856,28 +2699,24 @@
       <c r="F44" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G44" s="14" t="str">
+      <c r="G44" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECNA114_1301.xml</v>
       </c>
-      <c r="H44" s="14" t="str">
+      <c r="H44" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECNA114_1301.modelspec</v>
       </c>
-      <c r="I44" s="14" t="str">
+      <c r="I44" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECNA114_1301.py</v>
       </c>
-      <c r="J44" s="14" t="str">
+      <c r="J44" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A44,".py"),_xlfn.CONCAT(A44,".py"))</f>
         <v>iECNA114_1301.py</v>
       </c>
-      <c r="K44" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECNA114_1301.modelspec</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A45" s="4" t="s">
         <v>79</v>
       </c>
@@ -2896,28 +2735,24 @@
       <c r="F45" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G45" s="14" t="str">
+      <c r="G45" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECO103_1326.xml</v>
       </c>
-      <c r="H45" s="14" t="str">
+      <c r="H45" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECO103_1326.modelspec</v>
       </c>
-      <c r="I45" s="14" t="str">
+      <c r="I45" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECO103_1326.py</v>
       </c>
-      <c r="J45" s="14" t="str">
+      <c r="J45" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECO103_1326.py</v>
       </c>
-      <c r="K45" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECO103_1326.modelspec</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A46" s="4" t="s">
         <v>81</v>
       </c>
@@ -2936,28 +2771,24 @@
       <c r="F46" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G46" s="14" t="str">
+      <c r="G46" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A46,".xml"),_xlfn.CONCAT(A46,".xml"))</f>
         <v>iECO111_1330.xml</v>
       </c>
-      <c r="H46" s="14" t="str">
+      <c r="H46" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECO111_1330.modelspec</v>
       </c>
-      <c r="I46" s="14" t="str">
+      <c r="I46" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECO111_1330.py</v>
       </c>
-      <c r="J46" s="14" t="str">
+      <c r="J46" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A46,".py"),_xlfn.CONCAT(A46,".py"))</f>
         <v>iECO111_1330.py</v>
       </c>
-      <c r="K46" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECO111_1330.modelspec</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A47" s="4" t="s">
         <v>83</v>
       </c>
@@ -2976,28 +2807,24 @@
       <c r="F47" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G47" s="14" t="str">
+      <c r="G47" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A47,".xml"),_xlfn.CONCAT(A47,".xml"))</f>
         <v>iECO26_1355.xml</v>
       </c>
-      <c r="H47" s="14" t="str">
+      <c r="H47" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECO26_1355.modelspec</v>
       </c>
-      <c r="I47" s="14" t="str">
+      <c r="I47" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECO26_1355.py</v>
       </c>
-      <c r="J47" s="14" t="str">
+      <c r="J47" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECO26_1355.py</v>
       </c>
-      <c r="K47" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECO26_1355.modelspec</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A48" s="4" t="s">
         <v>85</v>
       </c>
@@ -3016,28 +2843,24 @@
       <c r="F48" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G48" s="14" t="str">
+      <c r="G48" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECOK1_1307.xml</v>
       </c>
-      <c r="H48" s="14" t="str">
+      <c r="H48" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECOK1_1307.modelspec</v>
       </c>
-      <c r="I48" s="14" t="str">
+      <c r="I48" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECOK1_1307.py</v>
       </c>
-      <c r="J48" s="14" t="str">
+      <c r="J48" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECOK1_1307.py</v>
       </c>
-      <c r="K48" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECOK1_1307.modelspec</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A49" s="4" t="s">
         <v>87</v>
       </c>
@@ -3056,28 +2879,24 @@
       <c r="F49" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G49" s="14" t="str">
+      <c r="G49" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A49,".xml"),_xlfn.CONCAT(A49,".xml"))</f>
         <v>iEcolC_1368.xml</v>
       </c>
-      <c r="H49" s="14" t="str">
+      <c r="H49" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A49,".modelspec"),_xlfn.CONCAT(A49,".modelspec"))</f>
         <v>iEcolC_1368.modelspec</v>
       </c>
-      <c r="I49" s="14" t="str">
+      <c r="I49" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A49,".py"),_xlfn.CONCAT(A49,".py"))</f>
         <v>iEcolC_1368.py</v>
       </c>
-      <c r="J49" s="14" t="str">
+      <c r="J49" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEcolC_1368.py</v>
       </c>
-      <c r="K49" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iEcolC_1368.modelspec</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A50" s="4" t="s">
         <v>88</v>
       </c>
@@ -3096,28 +2915,24 @@
       <c r="F50" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G50" s="14" t="str">
+      <c r="G50" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECP_1309.xml</v>
       </c>
-      <c r="H50" s="14" t="str">
+      <c r="H50" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECP_1309.modelspec</v>
       </c>
-      <c r="I50" s="14" t="str">
+      <c r="I50" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECP_1309.py</v>
       </c>
-      <c r="J50" s="14" t="str">
+      <c r="J50" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECP_1309.py</v>
       </c>
-      <c r="K50" s="13" t="str">
-        <f t="shared" si="4"/>
-        <v>iECP_1309.modelspec</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A51" s="4" t="s">
         <v>90</v>
       </c>
@@ -3136,27 +2951,24 @@
       <c r="F51" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G51" s="14" t="str">
+      <c r="G51" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECs_1301.xml</v>
       </c>
-      <c r="H51" s="14" t="str">
+      <c r="H51" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A51,".modelspec"),_xlfn.CONCAT(A51,".modelspec"))</f>
         <v>iECs_1301.modelspec</v>
       </c>
-      <c r="I51" s="14" t="str">
+      <c r="I51" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECs_1301.py</v>
       </c>
-      <c r="J51" s="14" t="str">
+      <c r="J51" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECs_1301.py</v>
       </c>
-      <c r="K51" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A52" s="4" t="s">
         <v>92</v>
       </c>
@@ -3175,27 +2987,24 @@
       <c r="F52" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G52" s="14" t="str">
+      <c r="G52" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECS88_1305.xml</v>
       </c>
-      <c r="H52" s="14" t="str">
+      <c r="H52" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECS88_1305.modelspec</v>
       </c>
-      <c r="I52" s="14" t="str">
+      <c r="I52" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECS88_1305.py</v>
       </c>
-      <c r="J52" s="14" t="str">
+      <c r="J52" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECS88_1305.py</v>
       </c>
-      <c r="K52" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A53" s="4" t="s">
         <v>94</v>
       </c>
@@ -3214,27 +3023,24 @@
       <c r="F53" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G53" s="14" t="str">
+      <c r="G53" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECSE_1348.xml</v>
       </c>
-      <c r="H53" s="14" t="str">
+      <c r="H53" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iECSE_1348.modelspec</v>
       </c>
-      <c r="I53" s="14" t="str">
+      <c r="I53" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECSE_1348.py</v>
       </c>
-      <c r="J53" s="14" t="str">
+      <c r="J53" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECSE_1348.py</v>
       </c>
-      <c r="K53" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A54" s="4" t="s">
         <v>96</v>
       </c>
@@ -3253,27 +3059,24 @@
       <c r="F54" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G54" s="14" t="str">
+      <c r="G54" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECSF_1327.xml</v>
       </c>
-      <c r="H54" s="14" t="str">
+      <c r="H54" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A54,".modelspec"),_xlfn.CONCAT(A54,".modelspec"))</f>
         <v>iECSF_1327.modelspec</v>
       </c>
-      <c r="I54" s="14" t="str">
+      <c r="I54" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A54,".py"),_xlfn.CONCAT(A54,".py"))</f>
         <v>iECSF_1327.py</v>
       </c>
-      <c r="J54" s="14" t="str">
+      <c r="J54" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECSF_1327.py</v>
       </c>
-      <c r="K54" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A55" s="4" t="s">
         <v>98</v>
       </c>
@@ -3292,27 +3095,24 @@
       <c r="F55" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G55" s="14" t="str">
+      <c r="G55" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A55,".xml"),_xlfn.CONCAT(A55,".xml"))</f>
         <v>iEcSMS35_1347.xml</v>
       </c>
-      <c r="H55" s="14" t="str">
+      <c r="H55" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iEcSMS35_1347.modelspec</v>
       </c>
-      <c r="I55" s="14" t="str">
+      <c r="I55" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A55,".py"),_xlfn.CONCAT(A55,".py"))</f>
         <v>iEcSMS35_1347.py</v>
       </c>
-      <c r="J55" s="14" t="str">
+      <c r="J55" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEcSMS35_1347.py</v>
       </c>
-      <c r="K55" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
         <v>100</v>
       </c>
@@ -3331,27 +3131,24 @@
       <c r="F56" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G56" s="14" t="str">
+      <c r="G56" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECSP_1301.xml</v>
       </c>
-      <c r="H56" s="14" t="str">
+      <c r="H56" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A56,".modelspec"),_xlfn.CONCAT(A56,".modelspec"))</f>
         <v>iECSP_1301.modelspec</v>
       </c>
-      <c r="I56" s="14" t="str">
+      <c r="I56" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A56,".py"),_xlfn.CONCAT(A56,".py"))</f>
         <v>iECSP_1301.py</v>
       </c>
-      <c r="J56" s="14" t="str">
+      <c r="J56" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECSP_1301.py</v>
       </c>
-      <c r="K56" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A57" s="4" t="s">
         <v>102</v>
       </c>
@@ -3370,27 +3167,24 @@
       <c r="F57" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G57" s="14" t="str">
+      <c r="G57" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECUMN_1333.xml</v>
       </c>
-      <c r="H57" s="14" t="str">
+      <c r="H57" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A57,".modelspec"),_xlfn.CONCAT(A57,".modelspec"))</f>
         <v>iECUMN_1333.modelspec</v>
       </c>
-      <c r="I57" s="14" t="str">
+      <c r="I57" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECUMN_1333.py</v>
       </c>
-      <c r="J57" s="14" t="str">
+      <c r="J57" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A57,".py"),_xlfn.CONCAT(A57,".py"))</f>
         <v>iECUMN_1333.py</v>
       </c>
-      <c r="K57" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A58" s="4" t="s">
         <v>104</v>
       </c>
@@ -3409,27 +3203,24 @@
       <c r="F58" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G58" s="14" t="str">
+      <c r="G58" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iECW_1372.xml</v>
       </c>
-      <c r="H58" s="14" t="str">
+      <c r="H58" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A58,".modelspec"),_xlfn.CONCAT(A58,".modelspec"))</f>
         <v>iECW_1372.modelspec</v>
       </c>
-      <c r="I58" s="14" t="str">
+      <c r="I58" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iECW_1372.py</v>
       </c>
-      <c r="J58" s="14" t="str">
+      <c r="J58" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iECW_1372.py</v>
       </c>
-      <c r="K58" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A59" s="4" t="s">
         <v>105</v>
       </c>
@@ -3448,27 +3239,24 @@
       <c r="F59" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G59" s="14" t="str">
+      <c r="G59" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iEK1008.xml</v>
       </c>
-      <c r="H59" s="14" t="str">
+      <c r="H59" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A59,".modelspec"),_xlfn.CONCAT(A59,".modelspec"))</f>
         <v>iEK1008.modelspec</v>
       </c>
-      <c r="I59" s="14" t="str">
+      <c r="I59" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iEK1008.py</v>
       </c>
-      <c r="J59" s="14" t="str">
+      <c r="J59" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEK1008.py</v>
       </c>
-      <c r="K59" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A60" s="4" t="s">
         <v>107</v>
       </c>
@@ -3487,27 +3275,24 @@
       <c r="F60" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G60" s="14" t="str">
+      <c r="G60" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iEKO11_1354.xml</v>
       </c>
-      <c r="H60" s="14" t="str">
+      <c r="H60" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iEKO11_1354.modelspec</v>
       </c>
-      <c r="I60" s="14" t="str">
+      <c r="I60" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iEKO11_1354.py</v>
       </c>
-      <c r="J60" s="14" t="str">
+      <c r="J60" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iEKO11_1354.py</v>
       </c>
-      <c r="K60" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A61" s="4" t="s">
         <v>109</v>
       </c>
@@ -3526,27 +3311,24 @@
       <c r="F61" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G61" s="14" t="str">
+      <c r="G61" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iETEC_1333.xml</v>
       </c>
-      <c r="H61" s="14" t="str">
+      <c r="H61" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iETEC_1333.modelspec</v>
       </c>
-      <c r="I61" s="14" t="str">
+      <c r="I61" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A61,".py"),_xlfn.CONCAT(A61,".py"))</f>
         <v>iETEC_1333.py</v>
       </c>
-      <c r="J61" s="14" t="str">
+      <c r="J61" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iETEC_1333.py</v>
       </c>
-      <c r="K61" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A62" s="4" t="s">
         <v>111</v>
       </c>
@@ -3565,27 +3347,24 @@
       <c r="F62" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G62" s="14" t="str">
+      <c r="G62" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iG2583_1286.xml</v>
       </c>
-      <c r="H62" s="14" t="str">
+      <c r="H62" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iG2583_1286.modelspec</v>
       </c>
-      <c r="I62" s="14" t="str">
+      <c r="I62" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iG2583_1286.py</v>
       </c>
-      <c r="J62" s="14" t="str">
+      <c r="J62" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iG2583_1286.py</v>
       </c>
-      <c r="K62" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A63" s="4" t="s">
         <v>113</v>
       </c>
@@ -3604,27 +3383,24 @@
       <c r="F63" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G63" s="14" t="str">
+      <c r="G63" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iHN637.xml</v>
       </c>
-      <c r="H63" s="14" t="str">
+      <c r="H63" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iHN637.modelspec</v>
       </c>
-      <c r="I63" s="14" t="str">
+      <c r="I63" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iHN637.py</v>
       </c>
-      <c r="J63" s="14" t="str">
+      <c r="J63" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iHN637.py</v>
       </c>
-      <c r="K63" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A64" s="4" t="s">
         <v>115</v>
       </c>
@@ -3643,27 +3419,24 @@
       <c r="F64" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G64" s="14" t="str">
+      <c r="G64" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iIS312.xml</v>
       </c>
-      <c r="H64" s="14" t="str">
+      <c r="H64" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iIS312.modelspec</v>
       </c>
-      <c r="I64" s="14" t="str">
+      <c r="I64" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iIS312.py</v>
       </c>
-      <c r="J64" s="14" t="str">
+      <c r="J64" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iIS312.py</v>
       </c>
-      <c r="K64" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
+    </row>
+    <row r="65" spans="1:10" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A65" s="4" t="s">
         <v>117</v>
       </c>
@@ -3682,27 +3455,24 @@
       <c r="F65" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G65" s="14" t="str">
+      <c r="G65" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iIS312_Amastigote.xml</v>
       </c>
-      <c r="H65" s="14" t="str">
+      <c r="H65" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A65,".modelspec"),_xlfn.CONCAT(A65,".modelspec"))</f>
         <v>iIS312_Amastigote.modelspec</v>
       </c>
-      <c r="I65" s="14" t="str">
+      <c r="I65" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iIS312_Amastigote.py</v>
       </c>
-      <c r="J65" s="14" t="str">
+      <c r="J65" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iIS312_Amastigote.py</v>
       </c>
-      <c r="K65" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
+    </row>
+    <row r="66" spans="1:10" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A66" s="4" t="s">
         <v>118</v>
       </c>
@@ -3721,27 +3491,24 @@
       <c r="F66" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G66" s="14" t="str">
+      <c r="G66" s="13" t="str">
         <f t="shared" si="0"/>
         <v>iIS312_Epimastigote.xml</v>
       </c>
-      <c r="H66" s="14" t="str">
+      <c r="H66" s="13" t="str">
         <f t="shared" si="1"/>
         <v>iIS312_Epimastigote.modelspec</v>
       </c>
-      <c r="I66" s="14" t="str">
+      <c r="I66" s="13" t="str">
         <f t="shared" si="2"/>
         <v>iIS312_Epimastigote.py</v>
       </c>
-      <c r="J66" s="14" t="str">
+      <c r="J66" s="13" t="str">
         <f t="shared" si="3"/>
         <v>iIS312_Epimastigote.py</v>
       </c>
-      <c r="K66" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" ht="29.5" x14ac:dyDescent="0.4">
+    </row>
+    <row r="67" spans="1:10" ht="29.5" x14ac:dyDescent="0.4">
       <c r="A67" s="4" t="s">
         <v>119</v>
       </c>
@@ -3760,27 +3527,24 @@
       <c r="F67" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G67" s="14" t="str">
-        <f t="shared" ref="G67:G109" si="5">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A67,".xml"),_xlfn.CONCAT(A67,".xml"))</f>
+      <c r="G67" s="13" t="str">
+        <f t="shared" ref="G67:G109" si="4">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A67,".xml"),_xlfn.CONCAT(A67,".xml"))</f>
         <v>iIS312_Trypomastigote.xml</v>
       </c>
-      <c r="H67" s="14" t="str">
-        <f t="shared" ref="H67:H108" si="6">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A67,".modelspec"),_xlfn.CONCAT(A67,".modelspec"))</f>
+      <c r="H67" s="13" t="str">
+        <f t="shared" ref="H67:H108" si="5">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A67,".modelspec"),_xlfn.CONCAT(A67,".modelspec"))</f>
         <v>iIS312_Trypomastigote.modelspec</v>
       </c>
-      <c r="I67" s="14" t="str">
-        <f t="shared" ref="I67:I109" si="7">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A67,".py"),_xlfn.CONCAT(A67,".py"))</f>
+      <c r="I67" s="13" t="str">
+        <f t="shared" ref="I67:I109" si="6">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A67,".py"),_xlfn.CONCAT(A67,".py"))</f>
         <v>iIS312_Trypomastigote.py</v>
       </c>
-      <c r="J67" s="14" t="str">
-        <f t="shared" ref="J67:J109" si="8">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A67,".py"),_xlfn.CONCAT(A67,".py"))</f>
+      <c r="J67" s="13" t="str">
+        <f t="shared" ref="J67:J109" si="7">HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A67,".py"),_xlfn.CONCAT(A67,".py"))</f>
         <v>iIS312_Trypomastigote.py</v>
       </c>
-      <c r="K67" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A68" s="4" t="s">
         <v>120</v>
       </c>
@@ -3799,27 +3563,24 @@
       <c r="F68" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G68" s="14" t="str">
+      <c r="G68" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A68,".xml"),_xlfn.CONCAT(A68,".xml"))</f>
         <v>iIT341.xml</v>
       </c>
-      <c r="H68" s="14" t="str">
+      <c r="H68" s="13" t="str">
+        <f t="shared" si="5"/>
+        <v>iIT341.modelspec</v>
+      </c>
+      <c r="I68" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iIT341.modelspec</v>
-      </c>
-      <c r="I68" s="14" t="str">
+        <v>iIT341.py</v>
+      </c>
+      <c r="J68" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iIT341.py</v>
       </c>
-      <c r="J68" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iIT341.py</v>
-      </c>
-      <c r="K68" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A69" s="4" t="s">
         <v>122</v>
       </c>
@@ -3838,27 +3599,24 @@
       <c r="F69" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G69" s="14" t="str">
+      <c r="G69" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iJB785.xml</v>
+      </c>
+      <c r="H69" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iJB785.xml</v>
-      </c>
-      <c r="H69" s="14" t="str">
+        <v>iJB785.modelspec</v>
+      </c>
+      <c r="I69" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iJB785.modelspec</v>
-      </c>
-      <c r="I69" s="14" t="str">
+        <v>iJB785.py</v>
+      </c>
+      <c r="J69" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iJB785.py</v>
       </c>
-      <c r="J69" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iJB785.py</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A70" s="4" t="s">
         <v>124</v>
       </c>
@@ -3877,27 +3635,24 @@
       <c r="F70" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G70" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G70" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>iJN1463.xml</v>
       </c>
-      <c r="H70" s="14" t="str">
+      <c r="H70" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A70,".modelspec"),_xlfn.CONCAT(A70,".modelspec"))</f>
         <v>iJN1463.modelspec</v>
       </c>
-      <c r="I70" s="14" t="str">
+      <c r="I70" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>iJN1463.py</v>
+      </c>
+      <c r="J70" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iJN1463.py</v>
       </c>
-      <c r="J70" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iJN1463.py</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A71" s="4" t="s">
         <v>126</v>
       </c>
@@ -3916,27 +3671,24 @@
       <c r="F71" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G71" s="14" t="str">
+      <c r="G71" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iJN678.xml</v>
+      </c>
+      <c r="H71" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iJN678.xml</v>
-      </c>
-      <c r="H71" s="14" t="str">
+        <v>iJN678.modelspec</v>
+      </c>
+      <c r="I71" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iJN678.modelspec</v>
-      </c>
-      <c r="I71" s="14" t="str">
-        <f t="shared" si="7"/>
         <v>iJN678.py</v>
       </c>
-      <c r="J71" s="14" t="str">
+      <c r="J71" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A71,".py"),_xlfn.CONCAT(A71,".py"))</f>
         <v>iJN678.py</v>
       </c>
-      <c r="K71" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A72" s="4" t="s">
         <v>128</v>
       </c>
@@ -3955,27 +3707,24 @@
       <c r="F72" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G72" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G72" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>iJN746.xml</v>
       </c>
-      <c r="H72" s="14" t="str">
+      <c r="H72" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A72,".modelspec"),_xlfn.CONCAT(A72,".modelspec"))</f>
         <v>iJN746.modelspec</v>
       </c>
-      <c r="I72" s="14" t="str">
+      <c r="I72" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>iJN746.py</v>
+      </c>
+      <c r="J72" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iJN746.py</v>
       </c>
-      <c r="J72" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iJN746.py</v>
-      </c>
-      <c r="K72" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A73" s="4" t="s">
         <v>129</v>
       </c>
@@ -3994,27 +3743,24 @@
       <c r="F73" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G73" s="14" t="str">
+      <c r="G73" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iJO1366.xml</v>
+      </c>
+      <c r="H73" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iJO1366.xml</v>
-      </c>
-      <c r="H73" s="14" t="str">
+        <v>iJO1366.modelspec</v>
+      </c>
+      <c r="I73" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iJO1366.modelspec</v>
-      </c>
-      <c r="I73" s="14" t="str">
+        <v>iJO1366.py</v>
+      </c>
+      <c r="J73" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iJO1366.py</v>
       </c>
-      <c r="J73" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iJO1366.py</v>
-      </c>
-      <c r="K73" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A74" s="4" t="s">
         <v>130</v>
       </c>
@@ -4033,27 +3779,24 @@
       <c r="F74" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G74" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G74" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>iJR904.xml</v>
       </c>
-      <c r="H74" s="14" t="str">
+      <c r="H74" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A74,".modelspec"),_xlfn.CONCAT(A74,".modelspec"))</f>
         <v>iJR904.modelspec</v>
       </c>
-      <c r="I74" s="14" t="str">
+      <c r="I74" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>iJR904.py</v>
+      </c>
+      <c r="J74" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iJR904.py</v>
       </c>
-      <c r="J74" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iJR904.py</v>
-      </c>
-      <c r="K74" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A75" s="4" t="s">
         <v>131</v>
       </c>
@@ -4072,27 +3815,24 @@
       <c r="F75" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G75" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G75" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>iLB1027_lipid.xml</v>
       </c>
-      <c r="H75" s="14" t="str">
+      <c r="H75" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A75,".modelspec"),_xlfn.CONCAT(A75,".modelspec"))</f>
         <v>iLB1027_lipid.modelspec</v>
       </c>
-      <c r="I75" s="14" t="str">
+      <c r="I75" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A75,".py"),_xlfn.CONCAT(A75,".py"))</f>
         <v>iLB1027_lipid.py</v>
       </c>
-      <c r="J75" s="14" t="str">
-        <f t="shared" si="8"/>
+      <c r="J75" s="13" t="str">
+        <f t="shared" si="7"/>
         <v>iLB1027_lipid.py</v>
       </c>
-      <c r="K75" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A76" s="4" t="s">
         <v>133</v>
       </c>
@@ -4111,27 +3851,24 @@
       <c r="F76" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G76" s="14" t="str">
+      <c r="G76" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iLF82_1304.xml</v>
+      </c>
+      <c r="H76" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iLF82_1304.xml</v>
-      </c>
-      <c r="H76" s="14" t="str">
+        <v>iLF82_1304.modelspec</v>
+      </c>
+      <c r="I76" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iLF82_1304.modelspec</v>
-      </c>
-      <c r="I76" s="14" t="str">
+        <v>iLF82_1304.py</v>
+      </c>
+      <c r="J76" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iLF82_1304.py</v>
       </c>
-      <c r="J76" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iLF82_1304.py</v>
-      </c>
-      <c r="K76" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A77" s="4" t="s">
         <v>135</v>
       </c>
@@ -4150,27 +3887,24 @@
       <c r="F77" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G77" s="14" t="str">
+      <c r="G77" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iLJ478.xml</v>
+      </c>
+      <c r="H77" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iLJ478.xml</v>
-      </c>
-      <c r="H77" s="14" t="str">
+        <v>iLJ478.modelspec</v>
+      </c>
+      <c r="I77" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iLJ478.modelspec</v>
-      </c>
-      <c r="I77" s="14" t="str">
+        <v>iLJ478.py</v>
+      </c>
+      <c r="J77" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iLJ478.py</v>
       </c>
-      <c r="J77" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iLJ478.py</v>
-      </c>
-      <c r="K77" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A78" s="4" t="s">
         <v>137</v>
       </c>
@@ -4189,27 +3923,24 @@
       <c r="F78" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G78" s="14" t="str">
+      <c r="G78" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iML1515.xml</v>
+      </c>
+      <c r="H78" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iML1515.xml</v>
-      </c>
-      <c r="H78" s="14" t="str">
+        <v>iML1515.modelspec</v>
+      </c>
+      <c r="I78" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iML1515.modelspec</v>
-      </c>
-      <c r="I78" s="14" t="str">
+        <v>iML1515.py</v>
+      </c>
+      <c r="J78" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iML1515.py</v>
       </c>
-      <c r="J78" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iML1515.py</v>
-      </c>
-      <c r="K78" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A79" s="4" t="s">
         <v>138</v>
       </c>
@@ -4228,27 +3959,24 @@
       <c r="F79" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G79" s="14" t="str">
+      <c r="G79" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iMM1415.xml</v>
+      </c>
+      <c r="H79" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iMM1415.xml</v>
-      </c>
-      <c r="H79" s="14" t="str">
+        <v>iMM1415.modelspec</v>
+      </c>
+      <c r="I79" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iMM1415.modelspec</v>
-      </c>
-      <c r="I79" s="14" t="str">
+        <v>iMM1415.py</v>
+      </c>
+      <c r="J79" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iMM1415.py</v>
       </c>
-      <c r="J79" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iMM1415.py</v>
-      </c>
-      <c r="K79" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A80" s="4" t="s">
         <v>140</v>
       </c>
@@ -4267,27 +3995,24 @@
       <c r="F80" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G80" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G80" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>iMM904.xml</v>
       </c>
-      <c r="H80" s="14" t="str">
+      <c r="H80" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A80,".modelspec"),_xlfn.CONCAT(A80,".modelspec"))</f>
         <v>iMM904.modelspec</v>
       </c>
-      <c r="I80" s="14" t="str">
+      <c r="I80" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>iMM904.py</v>
+      </c>
+      <c r="J80" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iMM904.py</v>
       </c>
-      <c r="J80" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iMM904.py</v>
-      </c>
-      <c r="K80" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A81" s="4" t="s">
         <v>142</v>
       </c>
@@ -4306,27 +4031,24 @@
       <c r="F81" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G81" s="14" t="str">
+      <c r="G81" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iND750.xml</v>
+      </c>
+      <c r="H81" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iND750.xml</v>
-      </c>
-      <c r="H81" s="14" t="str">
+        <v>iND750.modelspec</v>
+      </c>
+      <c r="I81" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iND750.modelspec</v>
-      </c>
-      <c r="I81" s="14" t="str">
+        <v>iND750.py</v>
+      </c>
+      <c r="J81" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iND750.py</v>
       </c>
-      <c r="J81" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iND750.py</v>
-      </c>
-      <c r="K81" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A82" s="4" t="s">
         <v>143</v>
       </c>
@@ -4345,27 +4067,24 @@
       <c r="F82" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G82" s="14" t="str">
+      <c r="G82" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iNF517.xml</v>
+      </c>
+      <c r="H82" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iNF517.xml</v>
-      </c>
-      <c r="H82" s="14" t="str">
+        <v>iNF517.modelspec</v>
+      </c>
+      <c r="I82" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iNF517.modelspec</v>
-      </c>
-      <c r="I82" s="14" t="str">
+        <v>iNF517.py</v>
+      </c>
+      <c r="J82" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iNF517.py</v>
       </c>
-      <c r="J82" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iNF517.py</v>
-      </c>
-      <c r="K82" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A83" s="4" t="s">
         <v>145</v>
       </c>
@@ -4384,27 +4103,24 @@
       <c r="F83" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G83" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G83" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>iNJ661.xml</v>
       </c>
-      <c r="H83" s="14" t="str">
+      <c r="H83" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A83,".modelspec"),_xlfn.CONCAT(A83,".modelspec"))</f>
         <v>iNJ661.modelspec</v>
       </c>
-      <c r="I83" s="14" t="str">
+      <c r="I83" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>iNJ661.py</v>
+      </c>
+      <c r="J83" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iNJ661.py</v>
       </c>
-      <c r="J83" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iNJ661.py</v>
-      </c>
-      <c r="K83" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A84" s="4" t="s">
         <v>146</v>
       </c>
@@ -4423,27 +4139,24 @@
       <c r="F84" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G84" s="14" t="str">
+      <c r="G84" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iNRG857_1313.xml</v>
+      </c>
+      <c r="H84" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iNRG857_1313.xml</v>
-      </c>
-      <c r="H84" s="14" t="str">
+        <v>iNRG857_1313.modelspec</v>
+      </c>
+      <c r="I84" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iNRG857_1313.modelspec</v>
-      </c>
-      <c r="I84" s="14" t="str">
+        <v>iNRG857_1313.py</v>
+      </c>
+      <c r="J84" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iNRG857_1313.py</v>
       </c>
-      <c r="J84" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iNRG857_1313.py</v>
-      </c>
-      <c r="K84" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A85" s="4" t="s">
         <v>148</v>
       </c>
@@ -4462,27 +4175,24 @@
       <c r="F85" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G85" s="14" t="str">
+      <c r="G85" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iPC815.xml</v>
+      </c>
+      <c r="H85" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iPC815.xml</v>
-      </c>
-      <c r="H85" s="14" t="str">
+        <v>iPC815.modelspec</v>
+      </c>
+      <c r="I85" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iPC815.modelspec</v>
-      </c>
-      <c r="I85" s="14" t="str">
+        <v>iPC815.py</v>
+      </c>
+      <c r="J85" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iPC815.py</v>
       </c>
-      <c r="J85" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iPC815.py</v>
-      </c>
-      <c r="K85" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A86" s="4" t="s">
         <v>150</v>
       </c>
@@ -4501,27 +4211,24 @@
       <c r="F86" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G86" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G86" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>iRC1080.xml</v>
       </c>
-      <c r="H86" s="14" t="str">
+      <c r="H86" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A86,".modelspec"),_xlfn.CONCAT(A86,".modelspec"))</f>
         <v>iRC1080.modelspec</v>
       </c>
-      <c r="I86" s="14" t="str">
+      <c r="I86" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>iRC1080.py</v>
+      </c>
+      <c r="J86" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iRC1080.py</v>
       </c>
-      <c r="J86" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iRC1080.py</v>
-      </c>
-      <c r="K86" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A87" s="4" t="s">
         <v>152</v>
       </c>
@@ -4540,27 +4247,24 @@
       <c r="F87" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G87" s="14" t="str">
+      <c r="G87" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A87,".xml"),_xlfn.CONCAT(A87,".xml"))</f>
         <v>iS_1188.xml</v>
       </c>
-      <c r="H87" s="14" t="str">
+      <c r="H87" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A87,".modelspec"),_xlfn.CONCAT(A87,".modelspec"))</f>
         <v>iS_1188.modelspec</v>
       </c>
-      <c r="I87" s="14" t="str">
+      <c r="I87" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>iS_1188.py</v>
+      </c>
+      <c r="J87" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iS_1188.py</v>
       </c>
-      <c r="J87" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iS_1188.py</v>
-      </c>
-      <c r="K87" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A88" s="4" t="s">
         <v>154</v>
       </c>
@@ -4579,27 +4283,24 @@
       <c r="F88" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G88" s="14" t="str">
+      <c r="G88" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A88,".xml"),_xlfn.CONCAT(A88,".xml"))</f>
         <v>iSB619.xml</v>
       </c>
-      <c r="H88" s="14" t="str">
+      <c r="H88" s="13" t="str">
+        <f t="shared" si="5"/>
+        <v>iSB619.modelspec</v>
+      </c>
+      <c r="I88" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iSB619.modelspec</v>
-      </c>
-      <c r="I88" s="14" t="str">
+        <v>iSB619.py</v>
+      </c>
+      <c r="J88" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iSB619.py</v>
       </c>
-      <c r="J88" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iSB619.py</v>
-      </c>
-      <c r="K88" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A89" s="4" t="s">
         <v>156</v>
       </c>
@@ -4618,27 +4319,24 @@
       <c r="F89" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G89" s="14" t="str">
+      <c r="G89" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iSbBS512_1146.xml</v>
+      </c>
+      <c r="H89" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iSbBS512_1146.xml</v>
-      </c>
-      <c r="H89" s="14" t="str">
+        <v>iSbBS512_1146.modelspec</v>
+      </c>
+      <c r="I89" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iSbBS512_1146.modelspec</v>
-      </c>
-      <c r="I89" s="14" t="str">
+        <v>iSbBS512_1146.py</v>
+      </c>
+      <c r="J89" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iSbBS512_1146.py</v>
       </c>
-      <c r="J89" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iSbBS512_1146.py</v>
-      </c>
-      <c r="K89" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A90" s="4" t="s">
         <v>158</v>
       </c>
@@ -4657,27 +4355,24 @@
       <c r="F90" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G90" s="14" t="str">
+      <c r="G90" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iSBO_1134.xml</v>
+      </c>
+      <c r="H90" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iSBO_1134.xml</v>
-      </c>
-      <c r="H90" s="14" t="str">
+        <v>iSBO_1134.modelspec</v>
+      </c>
+      <c r="I90" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iSBO_1134.modelspec</v>
-      </c>
-      <c r="I90" s="14" t="str">
+        <v>iSBO_1134.py</v>
+      </c>
+      <c r="J90" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iSBO_1134.py</v>
       </c>
-      <c r="J90" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iSBO_1134.py</v>
-      </c>
-      <c r="K90" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A91" s="4" t="s">
         <v>160</v>
       </c>
@@ -4696,27 +4391,24 @@
       <c r="F91" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G91" s="14" t="str">
+      <c r="G91" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iSDY_1059.xml</v>
+      </c>
+      <c r="H91" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iSDY_1059.xml</v>
-      </c>
-      <c r="H91" s="14" t="str">
+        <v>iSDY_1059.modelspec</v>
+      </c>
+      <c r="I91" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iSDY_1059.modelspec</v>
-      </c>
-      <c r="I91" s="14" t="str">
+        <v>iSDY_1059.py</v>
+      </c>
+      <c r="J91" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iSDY_1059.py</v>
       </c>
-      <c r="J91" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iSDY_1059.py</v>
-      </c>
-      <c r="K91" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A92" s="4" t="s">
         <v>162</v>
       </c>
@@ -4735,27 +4427,24 @@
       <c r="F92" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G92" s="14" t="str">
+      <c r="G92" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iSF_1195.xml</v>
+      </c>
+      <c r="H92" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iSF_1195.xml</v>
-      </c>
-      <c r="H92" s="14" t="str">
-        <f t="shared" si="6"/>
         <v>iSF_1195.modelspec</v>
       </c>
-      <c r="I92" s="14" t="str">
+      <c r="I92" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A92,".py"),_xlfn.CONCAT(A92,".py"))</f>
         <v>iSF_1195.py</v>
       </c>
-      <c r="J92" s="14" t="str">
-        <f t="shared" si="8"/>
+      <c r="J92" s="13" t="str">
+        <f t="shared" si="7"/>
         <v>iSF_1195.py</v>
       </c>
-      <c r="K92" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A93" s="4" t="s">
         <v>164</v>
       </c>
@@ -4774,27 +4463,24 @@
       <c r="F93" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G93" s="14" t="str">
+      <c r="G93" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iSFV_1184.xml</v>
+      </c>
+      <c r="H93" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iSFV_1184.xml</v>
-      </c>
-      <c r="H93" s="14" t="str">
+        <v>iSFV_1184.modelspec</v>
+      </c>
+      <c r="I93" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iSFV_1184.modelspec</v>
-      </c>
-      <c r="I93" s="14" t="str">
+        <v>iSFV_1184.py</v>
+      </c>
+      <c r="J93" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iSFV_1184.py</v>
       </c>
-      <c r="J93" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iSFV_1184.py</v>
-      </c>
-      <c r="K93" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A94" s="4" t="s">
         <v>166</v>
       </c>
@@ -4813,27 +4499,24 @@
       <c r="F94" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G94" s="14" t="str">
+      <c r="G94" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iSFxv_1172.xml</v>
+      </c>
+      <c r="H94" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iSFxv_1172.xml</v>
-      </c>
-      <c r="H94" s="14" t="str">
-        <f t="shared" si="6"/>
         <v>iSFxv_1172.modelspec</v>
       </c>
-      <c r="I94" s="14" t="str">
+      <c r="I94" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/odescripts/",A94,".py"),_xlfn.CONCAT(A94,".py"))</f>
         <v>iSFxv_1172.py</v>
       </c>
-      <c r="J94" s="14" t="str">
-        <f t="shared" si="8"/>
+      <c r="J94" s="13" t="str">
+        <f t="shared" si="7"/>
         <v>iSFxv_1172.py</v>
       </c>
-      <c r="K94" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A95" s="4" t="s">
         <v>168</v>
       </c>
@@ -4852,27 +4535,24 @@
       <c r="F95" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G95" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G95" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>iSSON_1240.xml</v>
       </c>
-      <c r="H95" s="14" t="str">
+      <c r="H95" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A95,".modelspec"),_xlfn.CONCAT(A95,".modelspec"))</f>
         <v>iSSON_1240.modelspec</v>
       </c>
-      <c r="I95" s="14" t="str">
+      <c r="I95" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>iSSON_1240.py</v>
+      </c>
+      <c r="J95" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iSSON_1240.py</v>
       </c>
-      <c r="J95" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iSSON_1240.py</v>
-      </c>
-      <c r="K95" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A96" s="4" t="s">
         <v>170</v>
       </c>
@@ -4891,27 +4571,24 @@
       <c r="F96" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G96" s="14" t="str">
+      <c r="G96" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iSynCJ816.xml</v>
+      </c>
+      <c r="H96" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iSynCJ816.xml</v>
-      </c>
-      <c r="H96" s="14" t="str">
+        <v>iSynCJ816.modelspec</v>
+      </c>
+      <c r="I96" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iSynCJ816.modelspec</v>
-      </c>
-      <c r="I96" s="14" t="str">
+        <v>iSynCJ816.py</v>
+      </c>
+      <c r="J96" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iSynCJ816.py</v>
       </c>
-      <c r="J96" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iSynCJ816.py</v>
-      </c>
-      <c r="K96" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A97" s="4" t="s">
         <v>171</v>
       </c>
@@ -4930,27 +4607,24 @@
       <c r="F97" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G97" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G97" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>iUMN146_1321.xml</v>
       </c>
-      <c r="H97" s="14" t="str">
+      <c r="H97" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A97,".modelspec"),_xlfn.CONCAT(A97,".modelspec"))</f>
         <v>iUMN146_1321.modelspec</v>
       </c>
-      <c r="I97" s="14" t="str">
+      <c r="I97" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>iUMN146_1321.py</v>
+      </c>
+      <c r="J97" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iUMN146_1321.py</v>
       </c>
-      <c r="J97" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iUMN146_1321.py</v>
-      </c>
-      <c r="K97" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A98" s="4" t="s">
         <v>173</v>
       </c>
@@ -4969,27 +4643,24 @@
       <c r="F98" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G98" s="14" t="str">
+      <c r="G98" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iUMNK88_1353.xml</v>
+      </c>
+      <c r="H98" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iUMNK88_1353.xml</v>
-      </c>
-      <c r="H98" s="14" t="str">
+        <v>iUMNK88_1353.modelspec</v>
+      </c>
+      <c r="I98" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iUMNK88_1353.modelspec</v>
-      </c>
-      <c r="I98" s="14" t="str">
+        <v>iUMNK88_1353.py</v>
+      </c>
+      <c r="J98" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iUMNK88_1353.py</v>
       </c>
-      <c r="J98" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iUMNK88_1353.py</v>
-      </c>
-      <c r="K98" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A99" s="4" t="s">
         <v>175</v>
       </c>
@@ -5008,27 +4679,24 @@
       <c r="F99" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G99" s="14" t="str">
+      <c r="G99" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iUTI89_1310.xml</v>
+      </c>
+      <c r="H99" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iUTI89_1310.xml</v>
-      </c>
-      <c r="H99" s="14" t="str">
+        <v>iUTI89_1310.modelspec</v>
+      </c>
+      <c r="I99" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iUTI89_1310.modelspec</v>
-      </c>
-      <c r="I99" s="14" t="str">
+        <v>iUTI89_1310.py</v>
+      </c>
+      <c r="J99" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iUTI89_1310.py</v>
       </c>
-      <c r="J99" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iUTI89_1310.py</v>
-      </c>
-      <c r="K99" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A100" s="4" t="s">
         <v>177</v>
       </c>
@@ -5047,27 +4715,24 @@
       <c r="F100" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G100" s="14" t="str">
+      <c r="G100" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iWFL_1372.xml</v>
+      </c>
+      <c r="H100" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iWFL_1372.xml</v>
-      </c>
-      <c r="H100" s="14" t="str">
+        <v>iWFL_1372.modelspec</v>
+      </c>
+      <c r="I100" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iWFL_1372.modelspec</v>
-      </c>
-      <c r="I100" s="14" t="str">
-        <f t="shared" si="7"/>
         <v>iWFL_1372.py</v>
       </c>
-      <c r="J100" s="14" t="str">
+      <c r="J100" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A100,".py"),_xlfn.CONCAT(A100,".py"))</f>
         <v>iWFL_1372.py</v>
       </c>
-      <c r="K100" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A101" s="4" t="s">
         <v>178</v>
       </c>
@@ -5086,27 +4751,24 @@
       <c r="F101" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G101" s="14" t="str">
+      <c r="G101" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A101,".xml"),_xlfn.CONCAT(A101,".xml"))</f>
         <v>iY75_1357.xml</v>
       </c>
-      <c r="H101" s="14" t="str">
+      <c r="H101" s="13" t="str">
+        <f t="shared" si="5"/>
+        <v>iY75_1357.modelspec</v>
+      </c>
+      <c r="I101" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iY75_1357.modelspec</v>
-      </c>
-      <c r="I101" s="14" t="str">
+        <v>iY75_1357.py</v>
+      </c>
+      <c r="J101" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iY75_1357.py</v>
       </c>
-      <c r="J101" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iY75_1357.py</v>
-      </c>
-      <c r="K101" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="102" spans="1:11" ht="32" x14ac:dyDescent="0.4">
+    </row>
+    <row r="102" spans="1:10" ht="32" x14ac:dyDescent="0.4">
       <c r="A102" s="4" t="s">
         <v>179</v>
       </c>
@@ -5125,27 +4787,24 @@
       <c r="F102" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G102" s="14" t="str">
+      <c r="G102" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iYL1228.xml</v>
+      </c>
+      <c r="H102" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iYL1228.xml</v>
-      </c>
-      <c r="H102" s="14" t="str">
+        <v>iYL1228.modelspec</v>
+      </c>
+      <c r="I102" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iYL1228.modelspec</v>
-      </c>
-      <c r="I102" s="14" t="str">
+        <v>iYL1228.py</v>
+      </c>
+      <c r="J102" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iYL1228.py</v>
       </c>
-      <c r="J102" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iYL1228.py</v>
-      </c>
-      <c r="K102" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A103" s="4" t="s">
         <v>181</v>
       </c>
@@ -5164,27 +4823,24 @@
       <c r="F103" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G103" s="14" t="str">
+      <c r="G103" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/blob/main/GSM/",A103,".xml"),_xlfn.CONCAT(A103,".xml"))</f>
         <v>iYO844.xml</v>
       </c>
-      <c r="H103" s="14" t="str">
+      <c r="H103" s="13" t="str">
+        <f t="shared" si="5"/>
+        <v>iYO844.modelspec</v>
+      </c>
+      <c r="I103" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iYO844.modelspec</v>
-      </c>
-      <c r="I103" s="14" t="str">
-        <f t="shared" si="7"/>
         <v>iYO844.py</v>
       </c>
-      <c r="J103" s="14" t="str">
+      <c r="J103" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/GSM-odescripts/",A103,".py"),_xlfn.CONCAT(A103,".py"))</f>
         <v>iYO844.py</v>
       </c>
-      <c r="K103" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A104" s="4" t="s">
         <v>183</v>
       </c>
@@ -5203,27 +4859,24 @@
       <c r="F104" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G104" s="14" t="str">
+      <c r="G104" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iYS1720.xml</v>
+      </c>
+      <c r="H104" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iYS1720.xml</v>
-      </c>
-      <c r="H104" s="14" t="str">
+        <v>iYS1720.modelspec</v>
+      </c>
+      <c r="I104" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iYS1720.modelspec</v>
-      </c>
-      <c r="I104" s="14" t="str">
+        <v>iYS1720.py</v>
+      </c>
+      <c r="J104" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iYS1720.py</v>
       </c>
-      <c r="J104" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iYS1720.py</v>
-      </c>
-      <c r="K104" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="105" spans="1:11" ht="32" x14ac:dyDescent="0.4">
+    </row>
+    <row r="105" spans="1:10" ht="32" x14ac:dyDescent="0.4">
       <c r="A105" s="4" t="s">
         <v>185</v>
       </c>
@@ -5242,27 +4895,24 @@
       <c r="F105" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G105" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G105" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>iYS854.xml</v>
       </c>
-      <c r="H105" s="14" t="str">
+      <c r="H105" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A105,".modelspec"),_xlfn.CONCAT(A105,".modelspec"))</f>
         <v>iYS854.modelspec</v>
       </c>
-      <c r="I105" s="14" t="str">
+      <c r="I105" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>iYS854.py</v>
+      </c>
+      <c r="J105" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iYS854.py</v>
       </c>
-      <c r="J105" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iYS854.py</v>
-      </c>
-      <c r="K105" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A106" s="4" t="s">
         <v>187</v>
       </c>
@@ -5281,27 +4931,24 @@
       <c r="F106" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G106" s="14" t="str">
+      <c r="G106" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>iZ_1308.xml</v>
+      </c>
+      <c r="H106" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>iZ_1308.xml</v>
-      </c>
-      <c r="H106" s="14" t="str">
+        <v>iZ_1308.modelspec</v>
+      </c>
+      <c r="I106" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>iZ_1308.modelspec</v>
-      </c>
-      <c r="I106" s="14" t="str">
+        <v>iZ_1308.py</v>
+      </c>
+      <c r="J106" s="13" t="str">
         <f t="shared" si="7"/>
         <v>iZ_1308.py</v>
       </c>
-      <c r="J106" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>iZ_1308.py</v>
-      </c>
-      <c r="K106" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A107" s="4" t="s">
         <v>189</v>
       </c>
@@ -5320,27 +4967,24 @@
       <c r="F107" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G107" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G107" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>RECON1.xml</v>
       </c>
-      <c r="H107" s="14" t="str">
+      <c r="H107" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A107,".modelspec"),_xlfn.CONCAT(A107,".modelspec"))</f>
         <v>RECON1.modelspec</v>
       </c>
-      <c r="I107" s="14" t="str">
+      <c r="I107" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>RECON1.py</v>
+      </c>
+      <c r="J107" s="13" t="str">
         <f t="shared" si="7"/>
         <v>RECON1.py</v>
       </c>
-      <c r="J107" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>RECON1.py</v>
-      </c>
-      <c r="K107" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.4">
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A108" s="4" t="s">
         <v>190</v>
       </c>
@@ -5359,27 +5003,24 @@
       <c r="F108" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G108" s="14" t="str">
+      <c r="G108" s="13" t="str">
+        <f t="shared" si="4"/>
+        <v>Recon3D.xml</v>
+      </c>
+      <c r="H108" s="13" t="str">
         <f t="shared" si="5"/>
-        <v>Recon3D.xml</v>
-      </c>
-      <c r="H108" s="14" t="str">
+        <v>Recon3D.modelspec</v>
+      </c>
+      <c r="I108" s="13" t="str">
         <f t="shared" si="6"/>
-        <v>Recon3D.modelspec</v>
-      </c>
-      <c r="I108" s="14" t="str">
+        <v>Recon3D.py</v>
+      </c>
+      <c r="J108" s="13" t="str">
         <f t="shared" si="7"/>
         <v>Recon3D.py</v>
       </c>
-      <c r="J108" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>Recon3D.py</v>
-      </c>
-      <c r="K108" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="109" spans="1:11" ht="32" x14ac:dyDescent="0.4">
+    </row>
+    <row r="109" spans="1:10" ht="32" x14ac:dyDescent="0.4">
       <c r="A109" s="4" t="s">
         <v>191</v>
       </c>
@@ -5398,24 +5039,21 @@
       <c r="F109" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="G109" s="14" t="str">
-        <f t="shared" si="5"/>
+      <c r="G109" s="13" t="str">
+        <f t="shared" si="4"/>
         <v>STM_v1_0.xml</v>
       </c>
-      <c r="H109" s="14" t="str">
+      <c r="H109" s="13" t="str">
         <f>HYPERLINK(_xlfn.CONCAT("https://github.com/mauriceling/kinmodre/tree/main/asm/",A109,".modelspec"),_xlfn.CONCAT(A109,".modelspec"))</f>
         <v>STM_v1_0.modelspec</v>
       </c>
-      <c r="I109" s="14" t="str">
+      <c r="I109" s="13" t="str">
+        <f t="shared" si="6"/>
+        <v>STM_v1_0.py</v>
+      </c>
+      <c r="J109" s="13" t="str">
         <f t="shared" si="7"/>
         <v>STM_v1_0.py</v>
-      </c>
-      <c r="J109" s="14" t="str">
-        <f t="shared" si="8"/>
-        <v>STM_v1_0.py</v>
-      </c>
-      <c r="K109" s="1" t="s">
-        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>